<commit_message>
Fund MSL stake with new Weapons sleeve capital instead of Saronic trim
- Saronic restored to $70M
- Weapons sleeve commitment $390M -> $405M (+$15M for the L3Harris
  Missile Solutions pre-IPO stake); holdco $840M -> $855M
- Updated size labels, IC size check target and build-tab notes

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UyuhDckU335yoju6PQ6QJg
</commit_message>
<xml_diff>
--- a/models/Leviathan_PE_HOLDCO_Model_IC_VLetalis_Faxon.xlsx
+++ b/models/Leviathan_PE_HOLDCO_Model_IC_VLetalis_Faxon.xlsx
@@ -62,18 +62,6 @@
           </rPr>
           <t xml:space="preserve">Microsoft Office User:
 PLACEHOLDER — no public valuation data found for Superior &amp; Grand Valley. $400M EV is an assumed mid-market forging mark; replace with actual data.</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="C12" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Trimmed $70M -&gt; $55M to fund the $15M L3Harris Missile Solutions pre-IPO stake inside the fixed $390M sleeve. Saronic was the largest position; trim keeps the sleeve at $390M.</t>
         </r>
       </text>
     </comment>
@@ -218,6 +206,28 @@
 </comments>
 </file>
 
+<file path=xl/comments3.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <authors>
+    <author>Unknown Author</author>
+  </authors>
+  <commentList>
+    <comment ref="B7" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Raised $390M -&gt; $405M: +$15M new commitment to fund the L3Harris Missile Solutions pre-IPO stake (IC, 9/2026). No existing Weapons position trimmed for it. Holdco $840M -&gt; $855M.</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/comments6.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <authors>
@@ -269,10 +279,10 @@
     <t xml:space="preserve">PURPOSE</t>
   </si>
   <si>
-    <t xml:space="preserve">Leviathan's core PE holdco is an $840M vehicle across THREE sub-funds: IQT-mirror deep-tech ($250M), Weapons ($390M), and Consumer/Value ($200M). All three sleeves are modeled bottom-up from individual holdings — IQT-mirror (nine In-Q-Tel names), Weapons (eleven physical-layer holdings, incl. a pre-IPO stake in L3Harris Missile Solutions (IPO Q1 2027), incl. The Ellwood Group and Superior &amp; Grand Valley for missile-procurement metal forging, and Faxon Machining for NGP / MOP / TLAM / BLU-136 warhead-case and missile machining), Consumer/Value (nine DTC/spending-cycle names) — each across four scenarios, 5/7/10-yr holds, gross-to-net waterfall, and PME, and roll up to a blended holdco return on the Holdco Summary tab. Start there for the top-down view; the sleeve tabs hold the detail.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Scope: Leviathan runs four vehicles (~$1.5B AUM total); this workbook models only the core PE holdco vehicle ($840M) and its equity targets — not the other three vehicles.</t>
+    <t xml:space="preserve">Leviathan's core PE holdco is an $855M vehicle across THREE sub-funds: IQT-mirror deep-tech ($250M), Weapons ($405M), and Consumer/Value ($200M). All three sleeves are modeled bottom-up from individual holdings — IQT-mirror (nine In-Q-Tel names), Weapons (eleven physical-layer holdings, incl. a pre-IPO stake in L3Harris Missile Solutions (IPO Q1 2027), incl. The Ellwood Group and Superior &amp; Grand Valley for missile-procurement metal forging, and Faxon Machining for NGP / MOP / TLAM / BLU-136 warhead-case and missile machining), Consumer/Value (nine DTC/spending-cycle names) — each across four scenarios, 5/7/10-yr holds, gross-to-net waterfall, and PME, and roll up to a blended holdco return on the Holdco Summary tab. Start there for the top-down view; the sleeve tabs hold the detail.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scope: Leviathan runs four vehicles (~$1.5B AUM total); this workbook models only the core PE holdco vehicle ($855M) and its equity targets — not the other three vehicles.</t>
   </si>
   <si>
     <t xml:space="preserve">THE DEFENSE-SUPERCYCLE THESIS (now wired into returns)</t>
@@ -333,7 +343,7 @@
     <t xml:space="preserve">LEVIATHAN CORE PE HOLDCO — IC SUMMARY</t>
   </si>
   <si>
-    <t xml:space="preserve">$840M tripartite holdco (IQT-mirror / Weapons / Consumer-Value). USD $M. Expected = probability-weighted across Base/Bull/Bear/TSMC-Shock (weights on Defense Supercycle tab). Every figure links live to the model — no inputs on this page.</t>
+    <t xml:space="preserve">$855M tripartite holdco (IQT-mirror / Weapons / Consumer-Value). USD $M. Expected = probability-weighted across Base/Bull/Bear/TSMC-Shock (weights on Defense Supercycle tab). Every figure links live to the model — no inputs on this page.</t>
   </si>
   <si>
     <t xml:space="preserve">HEADLINE — RECOMMENDED 7-YEAR VEHICLE (Expected case, net to LP)</t>
@@ -465,7 +475,7 @@
     <t xml:space="preserve">Status</t>
   </si>
   <si>
-    <t xml:space="preserve">Holdco size = $840M</t>
+    <t xml:space="preserve">Holdco size = $855M</t>
   </si>
   <si>
     <t xml:space="preserve">IQT-mirror deployed = committed</t>
@@ -501,7 +511,7 @@
     <t xml:space="preserve">• Six of nine IQT entry marks and most Weapons marks are estimates — see Assumptions col J / Weapons Sleeve col J. Confirm via primary diligence before IC vote.</t>
   </si>
   <si>
-    <t xml:space="preserve">LEVIATHAN — CORE PE HOLDCO ($840M) — TRIPARTITE ROLL-UP</t>
+    <t xml:space="preserve">LEVIATHAN — CORE PE HOLDCO ($855M) — TRIPARTITE ROLL-UP</t>
   </si>
   <si>
     <t xml:space="preserve">Three sub-funds rolled up to a blended holdco return. Blue = lever. All three sleeves — IQT-mirror, Weapons, Consumer/Value — flow in bottom-up.</t>
@@ -555,7 +565,7 @@
     <t xml:space="preserve">Ballast + near-term DPI engine</t>
   </si>
   <si>
-    <t xml:space="preserve">TOTAL (must = $840M)</t>
+    <t xml:space="preserve">TOTAL (must = $855M)</t>
   </si>
   <si>
     <t xml:space="preserve">IQT-mirror: Substrate, EUV Tech, ThinTronics, EdgeCortix, Syntiant, Infleqtion, Diraq, Mueon, DefendEye</t>
@@ -1467,7 +1477,7 @@
     <t xml:space="preserve">Read: sized by strategic function, the sleeve is ~53% TSMC-alternative packaging/substrates (the sovereign core), ~25% denied-environment edge AI, ~20% next-gen compute, ~3% adjacent autonomy — a deliberate overweight to the domestic fail-safe chokepoints that re-rate hardest in a Taiwan/TSMC shock.</t>
   </si>
   <si>
-    <t xml:space="preserve">WEAPONS SLEEVE — BOTTOM-UP ($390M)</t>
+    <t xml:space="preserve">WEAPONS SLEEVE — BOTTOM-UP ($405M)</t>
   </si>
   <si>
     <t xml:space="preserve">Physical-layer defense holdings. Blue = input. Most entry marks are estimates; several names are access-constrained (see flags). Proceeds use munitions/FMS-adjusted CAGRs (cols S:V).</t>
@@ -1632,7 +1642,7 @@
     <t xml:space="preserve">Pre-IPO = 22x 2027E EBIT IPO value less 15% discount — see MSL Build</t>
   </si>
   <si>
-    <t xml:space="preserve">TOTAL (=$390M)</t>
+    <t xml:space="preserve">TOTAL (=$405M)</t>
   </si>
   <si>
     <t xml:space="preserve">5-YEAR HOLD — GROSS PROCEEDS</t>
@@ -1668,7 +1678,7 @@
     <t xml:space="preserve">Check size ($M)</t>
   </si>
   <si>
-    <t xml:space="preserve">User input: sub-$10M minority stake. Funded inside the fixed $390M sleeve by trimming Superior &amp; Grand Valley $40M -&gt; $31M.</t>
+    <t xml:space="preserve">User input: sub-$10M minority stake. Funded inside the Weapons sleeve by trimming Superior &amp; Grand Valley $40M -&gt; $31M.</t>
   </si>
   <si>
     <t xml:space="preserve">Ownership %</t>
@@ -2031,7 +2041,7 @@
     <t xml:space="preserve">Sleeve Adj. Base CAGR = build 7-yr Base CAGR</t>
   </si>
   <si>
-    <t xml:space="preserve">Weapons sleeve still fully deployed ($390M)</t>
+    <t xml:space="preserve">Weapons sleeve fully deployed (= committed)</t>
   </si>
   <si>
     <t xml:space="preserve">Stake &lt; $10M (user constraint)</t>
@@ -2103,7 +2113,7 @@
     <t xml:space="preserve">Pre-IPO post-money used for the Weapons Sleeve entry mark.</t>
   </si>
   <si>
-    <t xml:space="preserve">Sized per IC discussion (9/2026). Funded by trimming Saronic $70M -&gt; $55M.</t>
+    <t xml:space="preserve">Sized per IC discussion (9/2026). Funded by +$15M NEW commitment to the Weapons sleeve ($390M -&gt; $405M; holdco $840M -&gt; $855M) — no existing position trimmed.</t>
   </si>
   <si>
     <t xml:space="preserve">Check / entry valuation.</t>
@@ -2343,7 +2353,7 @@
     <t xml:space="preserve">PME, DPI &amp; PROBABILITY PRESSURE TEST</t>
   </si>
   <si>
-    <t xml:space="preserve">DPI/TVPI, KS-PME &amp; Direct Alpha vs SPX/NDX, and Expected Net IRR sensitivity to the TSMC-Shock probability. Rows 11-69 = IQT-mirror sleeve ($250M) only; rows 72+ = total $840M holdco (all three sleeves) — ties to IC Summary headline.</t>
+    <t xml:space="preserve">DPI/TVPI, KS-PME &amp; Direct Alpha vs SPX/NDX, and Expected Net IRR sensitivity to the TSMC-Shock probability. Rows 11-69 = IQT-mirror sleeve ($250M) only; rows 72+ = total $855M holdco (all three sleeves) — ties to IC Summary headline.</t>
   </si>
   <si>
     <t xml:space="preserve">PUBLIC-MARKET BENCHMARK ASSUMPTIONS (blue = lever)</t>
@@ -2418,7 +2428,7 @@
     <t xml:space="preserve">shock excluded</t>
   </si>
   <si>
-    <t xml:space="preserve">TOTAL HOLDCO ($840M) — DPI &amp; PME BY HOLD (Expected, probability-weighted)</t>
+    <t xml:space="preserve">TOTAL HOLDCO ($855M) — DPI &amp; PME BY HOLD (Expected, probability-weighted)</t>
   </si>
   <si>
     <t xml:space="preserve">5-yr</t>
@@ -2433,16 +2443,16 @@
     <t xml:space="preserve">Net KS-PME vs Defense+Semis basket</t>
   </si>
   <si>
-    <t xml:space="preserve">Links to Holdco Summary roll-ups (rows 38-44 / 59-65 / 80-86). Holdco = IQT-mirror + Weapons + Consumer/Value, 2%/8%/20% on $840M.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOTAL HOLDCO ($840M) — TSMC-SHOCK PROBABILITY PRESSURE TEST</t>
+    <t xml:space="preserve">Links to Holdco Summary roll-ups (rows 38-44 / 59-65 / 80-86). Holdco = IQT-mirror + Weapons + Consumer/Value, 2%/8%/20% on $855M.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOTAL HOLDCO ($855M) — TSMC-SHOCK PROBABILITY PRESSURE TEST</t>
   </si>
   <si>
     <t xml:space="preserve">Expected holdco Net IRR to LP as the TSMC-Shock probability varies (all three sleeves). Base/Bull/Bear keep their current relative weights; shock takes the remainder.</t>
   </si>
   <si>
-    <t xml:space="preserve">WEAPONS BOOK SLEEVE ($390M) — DPI &amp; PME BY HOLD (Expected, probability-weighted)</t>
+    <t xml:space="preserve">WEAPONS BOOK SLEEVE ($405M) — DPI &amp; PME BY HOLD (Expected, probability-weighted)</t>
   </si>
   <si>
     <t xml:space="preserve">Gross = sleeve proceeds from Weapons Sleeve tab. Net = gross × holdco expected net/gross ratio (pro-rata allocation of carry + fees; fees/carry are charged at holdco level).</t>
@@ -2648,15 +2658,15 @@
     </font>
     <font>
       <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
       <color rgb="FF0000FF"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
     </font>
     <font>
       <b val="true"/>
@@ -3312,11 +3322,11 @@
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="17" fillId="4" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="171" fontId="18" fillId="4" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="172" fontId="17" fillId="4" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="172" fontId="18" fillId="4" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3332,7 +3342,7 @@
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="174" fontId="17" fillId="4" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="174" fontId="18" fillId="4" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3452,7 +3462,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="172" fontId="17" fillId="3" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="172" fontId="18" fillId="3" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3508,7 +3518,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="173" fontId="17" fillId="13" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="173" fontId="18" fillId="13" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3520,7 +3530,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="173" fontId="17" fillId="4" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="173" fontId="18" fillId="4" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3528,7 +3538,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="17" fillId="4" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="18" fillId="4" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3536,7 +3546,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="17" fillId="4" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="169" fontId="18" fillId="4" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3560,7 +3570,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="176" fontId="17" fillId="4" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="176" fontId="18" fillId="4" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3612,7 +3622,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="13" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="18" fillId="13" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3620,7 +3630,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="17" fillId="4" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="171" fontId="18" fillId="4" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -4412,7 +4422,7 @@
       </c>
       <c r="E6" s="46" t="n">
         <f aca="false">C6/'Holdco Summary'!$B$9</f>
-        <v>0.157738095238095</v>
+        <v>0.154970760233918</v>
       </c>
       <c r="F6" s="92" t="n">
         <f aca="false">AVERAGE('Defense Supercycle'!G24,'Defense Supercycle'!G25,'Defense Supercycle'!G26)</f>
@@ -4443,7 +4453,7 @@
       </c>
       <c r="E7" s="46" t="n">
         <f aca="false">C7/'Holdco Summary'!$B$9</f>
-        <v>0.0738095238095238</v>
+        <v>0.0725146198830409</v>
       </c>
       <c r="F7" s="92" t="n">
         <f aca="false">AVERAGE('Defense Supercycle'!G27,'Defense Supercycle'!G28)</f>
@@ -4474,7 +4484,7 @@
       </c>
       <c r="E8" s="46" t="n">
         <f aca="false">C8/'Holdco Summary'!$B$9</f>
-        <v>0.0583333333333333</v>
+        <v>0.0573099415204678</v>
       </c>
       <c r="F8" s="92" t="n">
         <f aca="false">AVERAGE('Defense Supercycle'!G29,'Defense Supercycle'!G30,'Defense Supercycle'!G31)</f>
@@ -4505,7 +4515,7 @@
       </c>
       <c r="E9" s="46" t="n">
         <f aca="false">C9/'Holdco Summary'!$B$9</f>
-        <v>0.00773809523809524</v>
+        <v>0.00760233918128655</v>
       </c>
       <c r="F9" s="92" t="n">
         <f aca="false">AVERAGE('Defense Supercycle'!G32)</f>
@@ -5471,7 +5481,7 @@
       </c>
       <c r="B5" s="78" t="n">
         <f aca="false">'Holdco Summary'!$B$7</f>
-        <v>390</v>
+        <v>405</v>
       </c>
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
@@ -5669,11 +5679,11 @@
         <v>9250</v>
       </c>
       <c r="C12" s="79" t="n">
-        <v>55</v>
+        <v>70</v>
       </c>
       <c r="D12" s="46" t="n">
         <f aca="false">C12/B12</f>
-        <v>0.00594594594594595</v>
+        <v>0.00756756756756757</v>
       </c>
       <c r="E12" s="47" t="s">
         <v>426</v>
@@ -6373,7 +6383,7 @@
       <c r="B23" s="1"/>
       <c r="C23" s="50" t="n">
         <f aca="false">SUM(C12:C22)</f>
-        <v>390</v>
+        <v>405</v>
       </c>
       <c r="D23" s="1"/>
       <c r="E23" s="1"/>
@@ -6472,11 +6482,11 @@
       </c>
       <c r="B27" s="91" t="n">
         <f aca="false">C12</f>
-        <v>55</v>
+        <v>70</v>
       </c>
       <c r="C27" s="95" t="n">
         <f aca="false">B27*(1+S12)^5*'Weapons Sleeve'!$B$6</f>
-        <v>168.826054829529</v>
+        <v>214.869524328492</v>
       </c>
       <c r="D27" s="68" t="n">
         <f aca="false">C27/B27</f>
@@ -6488,7 +6498,7 @@
       </c>
       <c r="F27" s="95" t="n">
         <f aca="false">B27*(1+T12)^5*'Weapons Sleeve'!$B$6</f>
-        <v>292.14081651392</v>
+        <v>371.81558465408</v>
       </c>
       <c r="G27" s="68" t="n">
         <f aca="false">F27/B27</f>
@@ -6500,7 +6510,7 @@
       </c>
       <c r="I27" s="95" t="n">
         <f aca="false">B27*(1+U12)^5*'Weapons Sleeve'!$B$6</f>
-        <v>53.18110853506</v>
+        <v>67.68504722644</v>
       </c>
       <c r="J27" s="68" t="n">
         <f aca="false">I27/B27</f>
@@ -6508,11 +6518,11 @@
       </c>
       <c r="K27" s="46" t="n">
         <f aca="false">(I27/B27)^(1/5)-1</f>
-        <v>-0.00670342208525587</v>
+        <v>-0.00670342208525598</v>
       </c>
       <c r="L27" s="96" t="n">
         <f aca="false">B27*(1+V12)^5*'Weapons Sleeve'!$B$6</f>
-        <v>267.313907851217</v>
+        <v>340.217700901549</v>
       </c>
       <c r="M27" s="69" t="n">
         <f aca="false">L27/B27</f>
@@ -7109,55 +7119,55 @@
       </c>
       <c r="B38" s="97" t="n">
         <f aca="false">SUM(B27:B37)</f>
-        <v>390</v>
+        <v>405</v>
       </c>
       <c r="C38" s="97" t="n">
         <f aca="false">SUM(C27:C37)</f>
-        <v>915.68570629413</v>
+        <v>961.729175793093</v>
       </c>
       <c r="D38" s="98" t="n">
         <f aca="false">C38/B38</f>
-        <v>2.34791206742085</v>
+        <v>2.37463994022986</v>
       </c>
       <c r="E38" s="99" t="n">
         <f aca="false">(C38/B38)^(1/5)-1</f>
-        <v>0.186141130155831</v>
+        <v>0.188829446220983</v>
       </c>
       <c r="F38" s="97" t="n">
         <f aca="false">SUM(F27:F37)</f>
-        <v>1518.01135428847</v>
+        <v>1597.68612242863</v>
       </c>
       <c r="G38" s="98" t="n">
         <f aca="false">F38/B38</f>
-        <v>3.89233680586787</v>
+        <v>3.94490400599662</v>
       </c>
       <c r="H38" s="99" t="n">
         <f aca="false">(F38/B38)^(1/5)-1</f>
-        <v>0.312327055698143</v>
+        <v>0.315852736366111</v>
       </c>
       <c r="I38" s="97" t="n">
         <f aca="false">SUM(I27:I37)</f>
-        <v>433.967166232866</v>
+        <v>448.471104924246</v>
       </c>
       <c r="J38" s="98" t="n">
         <f aca="false">I38/B38</f>
-        <v>1.11273632367401</v>
+        <v>1.10733606154135</v>
       </c>
       <c r="K38" s="99" t="n">
         <f aca="false">(I38/B38)^(1/5)-1</f>
-        <v>0.0215942810159535</v>
+        <v>0.0206007630100915</v>
       </c>
       <c r="L38" s="100" t="n">
         <f aca="false">SUM(L27:L37)</f>
-        <v>1531.53081758509</v>
+        <v>1604.43461063542</v>
       </c>
       <c r="M38" s="101" t="n">
         <f aca="false">L38/B38</f>
-        <v>3.92700209637202</v>
+        <v>3.96156693984054</v>
       </c>
       <c r="N38" s="102" t="n">
         <f aca="false">(L38/B38)^(1/5)-1</f>
-        <v>0.314656299001643</v>
+        <v>0.31696247263922</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7261,11 +7271,11 @@
       </c>
       <c r="B43" s="91" t="n">
         <f aca="false">C12</f>
-        <v>55</v>
+        <v>70</v>
       </c>
       <c r="C43" s="95" t="n">
         <f aca="false">B43*(1+S12)^7*'Weapons Sleeve'!$B$7</f>
-        <v>261.486877295751</v>
+        <v>332.801480194592</v>
       </c>
       <c r="D43" s="68" t="n">
         <f aca="false">C43/B43</f>
@@ -7277,7 +7287,7 @@
       </c>
       <c r="F43" s="95" t="n">
         <f aca="false">B43*(1+T12)^7*'Weapons Sleeve'!$B$7</f>
-        <v>563.460884052639</v>
+        <v>717.132034248813</v>
       </c>
       <c r="G43" s="68" t="n">
         <f aca="false">F43/B43</f>
@@ -7289,7 +7299,7 @@
       </c>
       <c r="I43" s="95" t="n">
         <f aca="false">B43*(1+U12)^7*'Weapons Sleeve'!$B$7</f>
-        <v>51.8913510419793</v>
+        <v>66.0435376897918</v>
       </c>
       <c r="J43" s="68" t="n">
         <f aca="false">I43/B43</f>
@@ -7301,7 +7311,7 @@
       </c>
       <c r="L43" s="96" t="n">
         <f aca="false">B43*(1+V12)^7*'Weapons Sleeve'!$B$7</f>
-        <v>497.582175894592</v>
+        <v>633.286405684026</v>
       </c>
       <c r="M43" s="69" t="n">
         <f aca="false">L43/B43</f>
@@ -7898,55 +7908,55 @@
       </c>
       <c r="B54" s="97" t="n">
         <f aca="false">SUM(B43:B53)</f>
-        <v>390</v>
+        <v>405</v>
       </c>
       <c r="C54" s="97" t="n">
         <f aca="false">SUM(C43:C53)</f>
-        <v>1296.54096147776</v>
+        <v>1367.85556437661</v>
       </c>
       <c r="D54" s="98" t="n">
         <f aca="false">C54/B54</f>
-        <v>3.32446400378914</v>
+        <v>3.3774211466089</v>
       </c>
       <c r="E54" s="99" t="n">
         <f aca="false">(C54/B54)^(1/7)-1</f>
-        <v>0.187221251956986</v>
+        <v>0.189904683804596</v>
       </c>
       <c r="F54" s="97" t="n">
         <f aca="false">SUM(F43:F53)</f>
-        <v>2663.99206233137</v>
+        <v>2817.66321252754</v>
       </c>
       <c r="G54" s="98" t="n">
         <f aca="false">F54/B54</f>
-        <v>6.83074887777274</v>
+        <v>6.95719311735195</v>
       </c>
       <c r="H54" s="99" t="n">
         <f aca="false">(F54/B54)^(1/7)-1</f>
-        <v>0.315860226153021</v>
+        <v>0.319312637995968</v>
       </c>
       <c r="I54" s="97" t="n">
         <f aca="false">SUM(I43:I53)</f>
-        <v>451.571462496729</v>
+        <v>465.723649144541</v>
       </c>
       <c r="J54" s="98" t="n">
         <f aca="false">I54/B54</f>
-        <v>1.15787554486341</v>
+        <v>1.14993493615936</v>
       </c>
       <c r="K54" s="99" t="n">
         <f aca="false">(I54/B54)^(1/7)-1</f>
-        <v>0.0211617866038758</v>
+        <v>0.0201583997119177</v>
       </c>
       <c r="L54" s="100" t="n">
         <f aca="false">SUM(L43:L53)</f>
-        <v>2692.9346809097</v>
+        <v>2828.63891069913</v>
       </c>
       <c r="M54" s="101" t="n">
         <f aca="false">L54/B54</f>
-        <v>6.90496072028128</v>
+        <v>6.98429360666453</v>
       </c>
       <c r="N54" s="102" t="n">
         <f aca="false">(L54/B54)^(1/7)-1</f>
-        <v>0.317893066655618</v>
+        <v>0.32004557875878</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8050,11 +8060,11 @@
       </c>
       <c r="B59" s="91" t="n">
         <f aca="false">C12</f>
-        <v>55</v>
+        <v>70</v>
       </c>
       <c r="C59" s="95" t="n">
         <f aca="false">B59*(1+S12)^10*'Weapons Sleeve'!$B$8</f>
-        <v>502.058647689221</v>
+        <v>638.983733422645</v>
       </c>
       <c r="D59" s="68" t="n">
         <f aca="false">C59/B59</f>
@@ -8066,7 +8076,7 @@
       </c>
       <c r="F59" s="95" t="n">
         <f aca="false">B59*(1+T12)^10*'Weapons Sleeve'!$B$8</f>
-        <v>1503.34959770159</v>
+        <v>1913.35403343838</v>
       </c>
       <c r="G59" s="68" t="n">
         <f aca="false">F59/B59</f>
@@ -8078,7 +8088,7 @@
       </c>
       <c r="I59" s="95" t="n">
         <f aca="false">B59*(1+U12)^10*'Weapons Sleeve'!$B$8</f>
-        <v>49.8184578560453</v>
+        <v>63.4053099986031</v>
       </c>
       <c r="J59" s="68" t="n">
         <f aca="false">I59/B59</f>
@@ -8090,7 +8100,7 @@
       </c>
       <c r="L59" s="96" t="n">
         <f aca="false">B59*(1+V12)^10*'Weapons Sleeve'!$B$8</f>
-        <v>1258.68952507228</v>
+        <v>1601.96848645563</v>
       </c>
       <c r="M59" s="69" t="n">
         <f aca="false">L59/B59</f>
@@ -8687,55 +8697,55 @@
       </c>
       <c r="B70" s="97" t="n">
         <f aca="false">SUM(B59:B69)</f>
-        <v>390</v>
+        <v>405</v>
       </c>
       <c r="C70" s="97" t="n">
         <f aca="false">SUM(C59:C69)</f>
-        <v>2216.90031706174</v>
+        <v>2353.82540279516</v>
       </c>
       <c r="D70" s="98" t="n">
         <f aca="false">C70/B70</f>
-        <v>5.68435978733779</v>
+        <v>5.81191457480287</v>
       </c>
       <c r="E70" s="99" t="n">
         <f aca="false">(C70/B70)^(1/10)-1</f>
-        <v>0.189784086386249</v>
+        <v>0.192427332423751</v>
       </c>
       <c r="F70" s="97" t="n">
         <f aca="false">SUM(F59:F69)</f>
-        <v>6362.82597009198</v>
+        <v>6772.83040582878</v>
       </c>
       <c r="G70" s="98" t="n">
         <f aca="false">F70/B70</f>
-        <v>16.3149383848512</v>
+        <v>16.7230380390834</v>
       </c>
       <c r="H70" s="99" t="n">
         <f aca="false">(F70/B70)^(1/10)-1</f>
-        <v>0.32208246088706</v>
+        <v>0.325352854416582</v>
       </c>
       <c r="I70" s="97" t="n">
         <f aca="false">SUM(I59:I69)</f>
-        <v>480.983029224514</v>
+        <v>494.569881367072</v>
       </c>
       <c r="J70" s="98" t="n">
         <f aca="false">I70/B70</f>
-        <v>1.2332898185244</v>
+        <v>1.22116020090635</v>
       </c>
       <c r="K70" s="99" t="n">
         <f aca="false">(I70/B70)^(1/10)-1</f>
-        <v>0.0211899089834458</v>
+        <v>0.0201810781311162</v>
       </c>
       <c r="L70" s="100" t="n">
         <f aca="false">SUM(L59:L69)</f>
-        <v>6448.54944420373</v>
+        <v>6791.82840558708</v>
       </c>
       <c r="M70" s="101" t="n">
         <f aca="false">L70/B70</f>
-        <v>16.534742164625</v>
+        <v>16.7699466804619</v>
       </c>
       <c r="N70" s="102" t="n">
         <f aca="false">(L70/B70)^(1/10)-1</f>
-        <v>0.323852935316205</v>
+        <v>0.325724151576512</v>
       </c>
     </row>
   </sheetData>
@@ -19058,15 +19068,15 @@
       </c>
       <c r="B74" s="175" t="n">
         <f aca="false">'Holdco Summary'!F38</f>
-        <v>2.26221016237823</v>
+        <v>2.27595084398942</v>
       </c>
       <c r="C74" s="175" t="n">
         <f aca="false">'Holdco Summary'!F59</f>
-        <v>3.42290649540101</v>
+        <v>3.45301348617188</v>
       </c>
       <c r="D74" s="175" t="n">
         <f aca="false">'Holdco Summary'!F80</f>
-        <v>6.83263713490145</v>
+        <v>6.9198197348059</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19075,15 +19085,15 @@
       </c>
       <c r="B75" s="175" t="n">
         <f aca="false">'Holdco Summary'!F39</f>
-        <v>2.26221016237823</v>
+        <v>2.27595084398942</v>
       </c>
       <c r="C75" s="175" t="n">
         <f aca="false">'Holdco Summary'!F60</f>
-        <v>3.42290649540101</v>
+        <v>3.45301348617188</v>
       </c>
       <c r="D75" s="175" t="n">
         <f aca="false">'Holdco Summary'!F81</f>
-        <v>6.83263713490145</v>
+        <v>6.9198197348059</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19092,15 +19102,15 @@
       </c>
       <c r="B76" s="176" t="n">
         <f aca="false">'Holdco Summary'!F40</f>
-        <v>0.177352715458623</v>
+        <v>0.178779502986822</v>
       </c>
       <c r="C76" s="176" t="n">
         <f aca="false">'Holdco Summary'!F61</f>
-        <v>0.192180867725363</v>
+        <v>0.193673267252674</v>
       </c>
       <c r="D76" s="176" t="n">
         <f aca="false">'Holdco Summary'!F82</f>
-        <v>0.211877816332995</v>
+        <v>0.213415331908954</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19109,15 +19119,15 @@
       </c>
       <c r="B77" s="178" t="n">
         <f aca="false">'Holdco Summary'!F41</f>
-        <v>1.47028138693269</v>
+        <v>1.47921188718093</v>
       </c>
       <c r="C77" s="178" t="n">
         <f aca="false">'Holdco Summary'!F62</f>
-        <v>1.87244706988098</v>
+        <v>1.88891662484182</v>
       </c>
       <c r="D77" s="178" t="n">
         <f aca="false">'Holdco Summary'!F83</f>
-        <v>2.88617976537917</v>
+        <v>2.92300663775207</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19126,15 +19136,15 @@
       </c>
       <c r="B78" s="178" t="n">
         <f aca="false">'Holdco Summary'!F42</f>
-        <v>1.22783704294971</v>
+        <v>1.23529493442159</v>
       </c>
       <c r="C78" s="178" t="n">
         <f aca="false">'Holdco Summary'!F63</f>
-        <v>1.454942838418</v>
+        <v>1.46774013529633</v>
       </c>
       <c r="D78" s="178" t="n">
         <f aca="false">'Holdco Summary'!F84</f>
-        <v>2.01281528691584</v>
+        <v>2.03849826500703</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19143,15 +19153,15 @@
       </c>
       <c r="B79" s="178" t="n">
         <f aca="false">'Holdco Summary'!F43</f>
-        <v>1.12471826308982</v>
+        <v>1.13154981031405</v>
       </c>
       <c r="C79" s="178" t="n">
         <f aca="false">'Holdco Summary'!F64</f>
-        <v>1.28679733581458</v>
+        <v>1.29811566880597</v>
       </c>
       <c r="D79" s="178" t="n">
         <f aca="false">'Holdco Summary'!F85</f>
-        <v>1.68892340222796</v>
+        <v>1.71047360756428</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19160,15 +19170,15 @@
       </c>
       <c r="B80" s="179" t="n">
         <f aca="false">'Holdco Summary'!F44</f>
-        <v>0.02378496996402</v>
+        <v>0.0250256547711496</v>
       </c>
       <c r="C80" s="179" t="n">
         <f aca="false">'Holdco Summary'!F65</f>
-        <v>0.0366790154133589</v>
+        <v>0.0379767541327605</v>
       </c>
       <c r="D80" s="179" t="n">
         <f aca="false">'Holdco Summary'!F86</f>
-        <v>0.0538067968112996</v>
+        <v>0.0551437668773511</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19177,15 +19187,15 @@
       </c>
       <c r="B81" s="181" t="n">
         <f aca="false">B77^(1/5)-1</f>
-        <v>0.0801401059253422</v>
+        <v>0.0814490853090109</v>
       </c>
       <c r="C81" s="181" t="n">
         <f aca="false">C77^(1/7)-1</f>
-        <v>0.0937439153443693</v>
+        <v>0.0951130892226371</v>
       </c>
       <c r="D81" s="181" t="n">
         <f aca="false">D77^(1/10)-1</f>
-        <v>0.111814510397243</v>
+        <v>0.113225075145829</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19231,15 +19241,15 @@
       </c>
       <c r="B87" s="185" t="n">
         <f aca="false">(((1-$A87)*('Defense Supercycle'!$B$17*'Holdco Summary'!B37+'Defense Supercycle'!$B$18*'Holdco Summary'!C37+'Defense Supercycle'!$B$19*'Holdco Summary'!D37)/('Defense Supercycle'!$B$17+'Defense Supercycle'!$B$18+'Defense Supercycle'!$B$19)+$A87*'Holdco Summary'!E37)/'Holdco Summary'!$B$9)^(1/5)-1</f>
-        <v>0.170807063973927</v>
+        <v>0.172041492331849</v>
       </c>
       <c r="C87" s="185" t="n">
         <f aca="false">(((1-$A87)*('Defense Supercycle'!$B$17*'Holdco Summary'!B58+'Defense Supercycle'!$B$18*'Holdco Summary'!C58+'Defense Supercycle'!$B$19*'Holdco Summary'!D58)/('Defense Supercycle'!$B$17+'Defense Supercycle'!$B$18+'Defense Supercycle'!$B$19)+$A87*'Holdco Summary'!E58)/'Holdco Summary'!$B$9)^(1/7)-1</f>
-        <v>0.18429576547191</v>
+        <v>0.185622386660826</v>
       </c>
       <c r="D87" s="185" t="n">
         <f aca="false">(((1-$A87)*('Defense Supercycle'!$B$17*'Holdco Summary'!B79+'Defense Supercycle'!$B$18*'Holdco Summary'!C79+'Defense Supercycle'!$B$19*'Holdco Summary'!D79)/('Defense Supercycle'!$B$17+'Defense Supercycle'!$B$18+'Defense Supercycle'!$B$19)+$A87*'Holdco Summary'!E79)/'Holdco Summary'!$B$9)^(1/10)-1</f>
-        <v>0.202684088385577</v>
+        <v>0.204103263202339</v>
       </c>
       <c r="E87" s="186" t="s">
         <v>719</v>
@@ -19251,15 +19261,15 @@
       </c>
       <c r="B88" s="185" t="n">
         <f aca="false">(((1-$A88)*('Defense Supercycle'!$B$17*'Holdco Summary'!B37+'Defense Supercycle'!$B$18*'Holdco Summary'!C37+'Defense Supercycle'!$B$19*'Holdco Summary'!D37)/('Defense Supercycle'!$B$17+'Defense Supercycle'!$B$18+'Defense Supercycle'!$B$19)+$A88*'Holdco Summary'!E37)/'Holdco Summary'!$B$9)^(1/5)-1</f>
-        <v>0.173005211773832</v>
+        <v>0.174304711633184</v>
       </c>
       <c r="C88" s="185" t="n">
         <f aca="false">(((1-$A88)*('Defense Supercycle'!$B$17*'Holdco Summary'!B58+'Defense Supercycle'!$B$18*'Holdco Summary'!C58+'Defense Supercycle'!$B$19*'Holdco Summary'!D58)/('Defense Supercycle'!$B$17+'Defense Supercycle'!$B$18+'Defense Supercycle'!$B$19)+$A88*'Holdco Summary'!E58)/'Holdco Summary'!$B$9)^(1/7)-1</f>
-        <v>0.186959181637902</v>
+        <v>0.188342511590328</v>
       </c>
       <c r="D88" s="185" t="n">
         <f aca="false">(((1-$A88)*('Defense Supercycle'!$B$17*'Holdco Summary'!B79+'Defense Supercycle'!$B$18*'Holdco Summary'!C79+'Defense Supercycle'!$B$19*'Holdco Summary'!D79)/('Defense Supercycle'!$B$17+'Defense Supercycle'!$B$18+'Defense Supercycle'!$B$19)+$A88*'Holdco Summary'!E79)/'Holdco Summary'!$B$9)^(1/10)-1</f>
-        <v>0.205819228650319</v>
+        <v>0.207279596577157</v>
       </c>
       <c r="E88" s="186" t="str">
         <f aca="false">IF(ABS($A88-'Defense Supercycle'!$B$20)&lt;0.0001,"current base case","")</f>
@@ -19272,15 +19282,15 @@
       </c>
       <c r="B89" s="185" t="n">
         <f aca="false">(((1-$A89)*('Defense Supercycle'!$B$17*'Holdco Summary'!B37+'Defense Supercycle'!$B$18*'Holdco Summary'!C37+'Defense Supercycle'!$B$19*'Holdco Summary'!D37)/('Defense Supercycle'!$B$17+'Defense Supercycle'!$B$18+'Defense Supercycle'!$B$19)+$A89*'Holdco Summary'!E37)/'Holdco Summary'!$B$9)^(1/5)-1</f>
-        <v>0.175187005183742</v>
+        <v>0.176550616781995</v>
       </c>
       <c r="C89" s="185" t="n">
         <f aca="false">(((1-$A89)*('Defense Supercycle'!$B$17*'Holdco Summary'!B58+'Defense Supercycle'!$B$18*'Holdco Summary'!C58+'Defense Supercycle'!$B$19*'Holdco Summary'!D58)/('Defense Supercycle'!$B$17+'Defense Supercycle'!$B$18+'Defense Supercycle'!$B$19)+$A89*'Holdco Summary'!E58)/'Holdco Summary'!$B$9)^(1/7)-1</f>
-        <v>0.189587214743112</v>
+        <v>0.191025783454299</v>
       </c>
       <c r="D89" s="185" t="n">
         <f aca="false">(((1-$A89)*('Defense Supercycle'!$B$17*'Holdco Summary'!B79+'Defense Supercycle'!$B$18*'Holdco Summary'!C79+'Defense Supercycle'!$B$19*'Holdco Summary'!D79)/('Defense Supercycle'!$B$17+'Defense Supercycle'!$B$18+'Defense Supercycle'!$B$19)+$A89*'Holdco Summary'!E79)/'Holdco Summary'!$B$9)^(1/10)-1</f>
-        <v>0.208882679587533</v>
+        <v>0.210382453298415</v>
       </c>
       <c r="E89" s="186" t="str">
         <f aca="false">IF(ABS($A89-'Defense Supercycle'!$B$20)&lt;0.0001,"current base case","")</f>
@@ -19293,15 +19303,15 @@
       </c>
       <c r="B90" s="185" t="n">
         <f aca="false">(((1-$A90)*('Defense Supercycle'!$B$17*'Holdco Summary'!B37+'Defense Supercycle'!$B$18*'Holdco Summary'!C37+'Defense Supercycle'!$B$19*'Holdco Summary'!D37)/('Defense Supercycle'!$B$17+'Defense Supercycle'!$B$18+'Defense Supercycle'!$B$19)+$A90*'Holdco Summary'!E37)/'Holdco Summary'!$B$9)^(1/5)-1</f>
-        <v>0.177352715458623</v>
+        <v>0.178779502986822</v>
       </c>
       <c r="C90" s="185" t="n">
         <f aca="false">(((1-$A90)*('Defense Supercycle'!$B$17*'Holdco Summary'!B58+'Defense Supercycle'!$B$18*'Holdco Summary'!C58+'Defense Supercycle'!$B$19*'Holdco Summary'!D58)/('Defense Supercycle'!$B$17+'Defense Supercycle'!$B$18+'Defense Supercycle'!$B$19)+$A90*'Holdco Summary'!E58)/'Holdco Summary'!$B$9)^(1/7)-1</f>
-        <v>0.192180867725362</v>
+        <v>0.193673267252674</v>
       </c>
       <c r="D90" s="185" t="n">
         <f aca="false">(((1-$A90)*('Defense Supercycle'!$B$17*'Holdco Summary'!B79+'Defense Supercycle'!$B$18*'Holdco Summary'!C79+'Defense Supercycle'!$B$19*'Holdco Summary'!D79)/('Defense Supercycle'!$B$17+'Defense Supercycle'!$B$18+'Defense Supercycle'!$B$19)+$A90*'Holdco Summary'!E79)/'Holdco Summary'!$B$9)^(1/10)-1</f>
-        <v>0.211877816332995</v>
+        <v>0.213415331908954</v>
       </c>
       <c r="E90" s="186" t="str">
         <f aca="false">IF(ABS($A90-'Defense Supercycle'!$B$20)&lt;0.0001,"current base case","")</f>
@@ -19314,15 +19324,15 @@
       </c>
       <c r="B91" s="185" t="n">
         <f aca="false">(((1-$A91)*('Defense Supercycle'!$B$17*'Holdco Summary'!B37+'Defense Supercycle'!$B$18*'Holdco Summary'!C37+'Defense Supercycle'!$B$19*'Holdco Summary'!D37)/('Defense Supercycle'!$B$17+'Defense Supercycle'!$B$18+'Defense Supercycle'!$B$19)+$A91*'Holdco Summary'!E37)/'Holdco Summary'!$B$9)^(1/5)-1</f>
-        <v>0.179502606918758</v>
+        <v>0.180991657699962</v>
       </c>
       <c r="C91" s="185" t="n">
         <f aca="false">(((1-$A91)*('Defense Supercycle'!$B$17*'Holdco Summary'!B58+'Defense Supercycle'!$B$18*'Holdco Summary'!C58+'Defense Supercycle'!$B$19*'Holdco Summary'!D58)/('Defense Supercycle'!$B$17+'Defense Supercycle'!$B$18+'Defense Supercycle'!$B$19)+$A91*'Holdco Summary'!E58)/'Holdco Summary'!$B$9)^(1/7)-1</f>
-        <v>0.194741100443027</v>
+        <v>0.196285981360697</v>
       </c>
       <c r="D91" s="185" t="n">
         <f aca="false">(((1-$A91)*('Defense Supercycle'!$B$17*'Holdco Summary'!B79+'Defense Supercycle'!$B$18*'Holdco Summary'!C79+'Defense Supercycle'!$B$19*'Holdco Summary'!D79)/('Defense Supercycle'!$B$17+'Defense Supercycle'!$B$18+'Defense Supercycle'!$B$19)+$A91*'Holdco Summary'!E79)/'Holdco Summary'!$B$9)^(1/10)-1</f>
-        <v>0.21480777734036</v>
+        <v>0.216381482898982</v>
       </c>
       <c r="E91" s="186" t="str">
         <f aca="false">IF(ABS($A91-'Defense Supercycle'!$B$20)&lt;0.0001,"current base case","")</f>
@@ -19335,15 +19345,15 @@
       </c>
       <c r="B92" s="185" t="n">
         <f aca="false">(((1-$A92)*('Defense Supercycle'!$B$17*'Holdco Summary'!B37+'Defense Supercycle'!$B$18*'Holdco Summary'!C37+'Defense Supercycle'!$B$19*'Holdco Summary'!D37)/('Defense Supercycle'!$B$17+'Defense Supercycle'!$B$18+'Defense Supercycle'!$B$19)+$A92*'Holdco Summary'!E37)/'Holdco Summary'!$B$9)^(1/5)-1</f>
-        <v>0.181636937188174</v>
+        <v>0.183187360891462</v>
       </c>
       <c r="C92" s="185" t="n">
         <f aca="false">(((1-$A92)*('Defense Supercycle'!$B$17*'Holdco Summary'!B58+'Defense Supercycle'!$B$18*'Holdco Summary'!C58+'Defense Supercycle'!$B$19*'Holdco Summary'!D58)/('Defense Supercycle'!$B$17+'Defense Supercycle'!$B$18+'Defense Supercycle'!$B$19)+$A92*'Holdco Summary'!E58)/'Holdco Summary'!$B$9)^(1/7)-1</f>
-        <v>0.197268832136125</v>
+        <v>0.198864900242989</v>
       </c>
       <c r="D92" s="185" t="n">
         <f aca="false">(((1-$A92)*('Defense Supercycle'!$B$17*'Holdco Summary'!B79+'Defense Supercycle'!$B$18*'Holdco Summary'!C79+'Defense Supercycle'!$B$19*'Holdco Summary'!D79)/('Defense Supercycle'!$B$17+'Defense Supercycle'!$B$18+'Defense Supercycle'!$B$19)+$A92*'Holdco Summary'!E79)/'Holdco Summary'!$B$9)^(1/10)-1</f>
-        <v>0.217675486175901</v>
+        <v>0.219283931794773</v>
       </c>
       <c r="E92" s="186" t="str">
         <f aca="false">IF(ABS($A92-'Defense Supercycle'!$B$20)&lt;0.0001,"current base case","")</f>
@@ -19356,15 +19366,15 @@
       </c>
       <c r="B93" s="185" t="n">
         <f aca="false">(((1-$A93)*('Defense Supercycle'!$B$17*'Holdco Summary'!B37+'Defense Supercycle'!$B$18*'Holdco Summary'!C37+'Defense Supercycle'!$B$19*'Holdco Summary'!D37)/('Defense Supercycle'!$B$17+'Defense Supercycle'!$B$18+'Defense Supercycle'!$B$19)+$A93*'Holdco Summary'!E37)/'Holdco Summary'!$B$9)^(1/5)-1</f>
-        <v>0.183755957422806</v>
+        <v>0.18536688531101</v>
       </c>
       <c r="C93" s="185" t="n">
         <f aca="false">(((1-$A93)*('Defense Supercycle'!$B$17*'Holdco Summary'!B58+'Defense Supercycle'!$B$18*'Holdco Summary'!C58+'Defense Supercycle'!$B$19*'Holdco Summary'!D58)/('Defense Supercycle'!$B$17+'Defense Supercycle'!$B$18+'Defense Supercycle'!$B$19)+$A93*'Holdco Summary'!E58)/'Holdco Summary'!$B$9)^(1/7)-1</f>
-        <v>0.199764943712947</v>
+        <v>0.20141095697163</v>
       </c>
       <c r="D93" s="185" t="n">
         <f aca="false">(((1-$A93)*('Defense Supercycle'!$B$17*'Holdco Summary'!B79+'Defense Supercycle'!$B$18*'Holdco Summary'!C79+'Defense Supercycle'!$B$19*'Holdco Summary'!D79)/('Defense Supercycle'!$B$17+'Defense Supercycle'!$B$18+'Defense Supercycle'!$B$19)+$A93*'Holdco Summary'!E79)/'Holdco Summary'!$B$9)^(1/10)-1</f>
-        <v>0.220483670849732</v>
+        <v>0.222125499610033</v>
       </c>
       <c r="E93" s="186" t="str">
         <f aca="false">IF(ABS($A93-'Defense Supercycle'!$B$20)&lt;0.0001,"current base case","")</f>
@@ -19377,15 +19387,15 @@
       </c>
       <c r="B94" s="188" t="n">
         <f aca="false">(((1-$A94)*('Defense Supercycle'!$B$17*'Holdco Summary'!B37+'Defense Supercycle'!$B$18*'Holdco Summary'!C37+'Defense Supercycle'!$B$19*'Holdco Summary'!D37)/('Defense Supercycle'!$B$17+'Defense Supercycle'!$B$18+'Defense Supercycle'!$B$19)+$A94*'Holdco Summary'!E37)/'Holdco Summary'!$B$9)^(1/5)-1</f>
-        <v>0.187949041372367</v>
+        <v>0.189678454222763</v>
       </c>
       <c r="C94" s="188" t="n">
         <f aca="false">(((1-$A94)*('Defense Supercycle'!$B$17*'Holdco Summary'!B58+'Defense Supercycle'!$B$18*'Holdco Summary'!C58+'Defense Supercycle'!$B$19*'Holdco Summary'!D58)/('Defense Supercycle'!$B$17+'Defense Supercycle'!$B$18+'Defense Supercycle'!$B$19)+$A94*'Holdco Summary'!E58)/'Holdco Summary'!$B$9)^(1/7)-1</f>
-        <v>0.204665651106906</v>
+        <v>0.206408023162932</v>
       </c>
       <c r="D94" s="188" t="n">
         <f aca="false">(((1-$A94)*('Defense Supercycle'!$B$17*'Holdco Summary'!B79+'Defense Supercycle'!$B$18*'Holdco Summary'!C79+'Defense Supercycle'!$B$19*'Holdco Summary'!D79)/('Defense Supercycle'!$B$17+'Defense Supercycle'!$B$18+'Defense Supercycle'!$B$19)+$A94*'Holdco Summary'!E79)/'Holdco Summary'!$B$9)^(1/10)-1</f>
-        <v>0.225931503286711</v>
+        <v>0.227636360519233</v>
       </c>
       <c r="E94" s="189" t="str">
         <f aca="false">IF(ABS($A94-'Defense Supercycle'!$B$20)&lt;0.0001,"current base case","")</f>
@@ -19441,15 +19451,15 @@
       </c>
       <c r="B101" s="194" t="n">
         <f aca="false">'Holdco Summary'!$B$7</f>
-        <v>390</v>
+        <v>405</v>
       </c>
       <c r="C101" s="194" t="n">
         <f aca="false">'Holdco Summary'!$B$7</f>
-        <v>390</v>
+        <v>405</v>
       </c>
       <c r="D101" s="194" t="n">
         <f aca="false">'Holdco Summary'!$B$7</f>
-        <v>390</v>
+        <v>405</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19458,15 +19468,15 @@
       </c>
       <c r="B102" s="194" t="n">
         <f aca="false">'Holdco Summary'!F29</f>
-        <v>1086.38610397717</v>
+        <v>1140.135517048</v>
       </c>
       <c r="C102" s="194" t="n">
         <f aca="false">'Holdco Summary'!F50</f>
-        <v>1721.1173697588</v>
+        <v>1814.10519107791</v>
       </c>
       <c r="D102" s="194" t="n">
         <f aca="false">'Holdco Summary'!F71</f>
-        <v>3627.74150621502</v>
+        <v>3845.38877575814</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19475,15 +19485,15 @@
       </c>
       <c r="B103" s="195" t="n">
         <f aca="false">B102/B101</f>
-        <v>2.78560539481325</v>
+        <v>2.81514942480987</v>
       </c>
       <c r="C103" s="195" t="n">
         <f aca="false">C102/C101</f>
-        <v>4.41312146092</v>
+        <v>4.47927207673558</v>
       </c>
       <c r="D103" s="195" t="n">
         <f aca="false">D102/D101</f>
-        <v>9.30190129798722</v>
+        <v>9.49478710063738</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19492,15 +19502,15 @@
       </c>
       <c r="B104" s="196" t="n">
         <f aca="false">B103^(1/B$100)-1</f>
-        <v>0.227393782460184</v>
+        <v>0.229986345820906</v>
       </c>
       <c r="C104" s="196" t="n">
         <f aca="false">C103^(1/C$100)-1</f>
-        <v>0.236250710960596</v>
+        <v>0.23888112043644</v>
       </c>
       <c r="D104" s="196" t="n">
         <f aca="false">D103^(1/D$100)-1</f>
-        <v>0.249847922597485</v>
+        <v>0.252415757426635</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19509,15 +19519,15 @@
       </c>
       <c r="B105" s="197" t="n">
         <f aca="false">'Holdco Summary'!F37/'Holdco Summary'!F31</f>
-        <v>0.867305820994541</v>
+        <v>0.866888959910737</v>
       </c>
       <c r="C105" s="197" t="n">
         <f aca="false">'Holdco Summary'!F58/'Holdco Summary'!F52</f>
-        <v>0.843463122332387</v>
+        <v>0.843078546393105</v>
       </c>
       <c r="D105" s="197" t="n">
         <f aca="false">'Holdco Summary'!F79/'Holdco Summary'!F73</f>
-        <v>0.823094303611507</v>
+        <v>0.822800372429311</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19526,15 +19536,15 @@
       </c>
       <c r="B106" s="198" t="n">
         <f aca="false">B102*B105</f>
-        <v>942.228991826979</v>
+        <v>988.370892531031</v>
       </c>
       <c r="C106" s="198" t="n">
         <f aca="false">C102*C105</f>
-        <v>1451.69903059726</v>
+        <v>1529.43316749815</v>
       </c>
       <c r="D106" s="198" t="n">
         <f aca="false">D102*D105</f>
-        <v>2985.97336874061</v>
+        <v>3163.98731682929</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19543,15 +19553,15 @@
       </c>
       <c r="B107" s="195" t="n">
         <f aca="false">B106/B101</f>
-        <v>2.41597177391533</v>
+        <v>2.44042195686674</v>
       </c>
       <c r="C107" s="195" t="n">
         <f aca="false">C106/C101</f>
-        <v>3.72230520665965</v>
+        <v>3.77637819135345</v>
       </c>
       <c r="D107" s="195" t="n">
         <f aca="false">D106/D101</f>
-        <v>7.65634197112976</v>
+        <v>7.81231436254146</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19560,15 +19570,15 @@
       </c>
       <c r="B108" s="196" t="n">
         <f aca="false">B107^(1/B$100)-1</f>
-        <v>0.192939368853149</v>
+        <v>0.195344216874197</v>
       </c>
       <c r="C108" s="196" t="n">
         <f aca="false">C107^(1/C$100)-1</f>
-        <v>0.206547901240161</v>
+        <v>0.209036339363743</v>
       </c>
       <c r="D108" s="196" t="n">
         <f aca="false">D107^(1/D$100)-1</f>
-        <v>0.225750650228251</v>
+        <v>0.228225107618929</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19577,15 +19587,15 @@
       </c>
       <c r="B109" s="200" t="n">
         <f aca="false">B107/(1+'Holdco Summary'!$B$21)^B$100</f>
-        <v>1.57021588427846</v>
+        <v>1.58610682557932</v>
       </c>
       <c r="C109" s="200" t="n">
         <f aca="false">C107/(1+'Holdco Summary'!$B$21)^C$100</f>
-        <v>2.03622841780141</v>
+        <v>2.06580819214981</v>
       </c>
       <c r="D109" s="200" t="n">
         <f aca="false">D107/(1+'Holdco Summary'!$B$21)^D$100</f>
-        <v>3.23412158989425</v>
+        <v>3.30000601360392</v>
       </c>
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19594,15 +19604,15 @@
       </c>
       <c r="B110" s="200" t="n">
         <f aca="false">B107/(1+'Holdco Summary'!$B$22)^B$100</f>
-        <v>1.31129268538676</v>
+        <v>1.32456326512064</v>
       </c>
       <c r="C110" s="200" t="n">
         <f aca="false">C107/(1+'Holdco Summary'!$B$22)^C$100</f>
-        <v>1.58220544736237</v>
+        <v>1.60518974504559</v>
       </c>
       <c r="D110" s="200" t="n">
         <f aca="false">D107/(1+'Holdco Summary'!$B$22)^D$100</f>
-        <v>2.25546913396384</v>
+        <v>2.30141678310309</v>
       </c>
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19611,15 +19621,15 @@
       </c>
       <c r="B111" s="200" t="n">
         <f aca="false">B107/(1+'Holdco Summary'!$B$23)^B$100</f>
-        <v>1.20116495912804</v>
+        <v>1.21332102126527</v>
       </c>
       <c r="C111" s="200" t="n">
         <f aca="false">C107/(1+'Holdco Summary'!$B$23)^C$100</f>
-        <v>1.39935240108194</v>
+        <v>1.41968043888754</v>
       </c>
       <c r="D111" s="200" t="n">
         <f aca="false">D107/(1+'Holdco Summary'!$B$23)^D$100</f>
-        <v>1.89253064010222</v>
+        <v>1.93108462983644</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19628,15 +19638,15 @@
       </c>
       <c r="B112" s="201" t="n">
         <f aca="false">B111^(1/B$100)-1</f>
-        <v>0.037338581611434</v>
+        <v>0.0394297538036497</v>
       </c>
       <c r="C112" s="201" t="n">
         <f aca="false">C111^(1/C$100)-1</f>
-        <v>0.0491720880349229</v>
+        <v>0.0513359472728199</v>
       </c>
       <c r="D112" s="201" t="n">
         <f aca="false">D111^(1/D$100)-1</f>
-        <v>0.0658701306332621</v>
+        <v>0.0680218327121123</v>
       </c>
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19645,15 +19655,15 @@
       </c>
       <c r="B113" s="201" t="n">
         <f aca="false">B109^(1/B$100)-1</f>
-        <v>0.0944397879386689</v>
+        <v>0.0966460705267862</v>
       </c>
       <c r="C113" s="201" t="n">
         <f aca="false">C109^(1/C$100)-1</f>
-        <v>0.106924680036845</v>
+        <v>0.109207650792424</v>
       </c>
       <c r="D113" s="201" t="n">
         <f aca="false">D109^(1/D$100)-1</f>
-        <v>0.12454188094335</v>
+        <v>0.126812025338467</v>
       </c>
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19717,23 +19727,23 @@
       </c>
       <c r="B118" s="194" t="n">
         <f aca="false">'Weapons Sleeve'!C54</f>
-        <v>1296.54096147776</v>
+        <v>1367.85556437661</v>
       </c>
       <c r="C118" s="194" t="n">
         <f aca="false">'Weapons Sleeve'!F54</f>
-        <v>2663.99206233137</v>
+        <v>2817.66321252754</v>
       </c>
       <c r="D118" s="194" t="n">
         <f aca="false">'Weapons Sleeve'!I54</f>
-        <v>451.571462496729</v>
+        <v>465.723649144541</v>
       </c>
       <c r="E118" s="206" t="n">
         <f aca="false">'Weapons Sleeve'!L54</f>
-        <v>2692.9346809097</v>
+        <v>2828.63891069913</v>
       </c>
       <c r="F118" s="207" t="n">
         <f aca="false">SUMPRODUCT(B117:E117,B118:E118)</f>
-        <v>1721.1173697588</v>
+        <v>1814.10519107791</v>
       </c>
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19742,23 +19752,23 @@
       </c>
       <c r="B119" s="208" t="n">
         <f aca="false">'Weapons Sleeve'!D54</f>
-        <v>3.32446400378914</v>
+        <v>3.3774211466089</v>
       </c>
       <c r="C119" s="208" t="n">
         <f aca="false">'Weapons Sleeve'!G54</f>
-        <v>6.83074887777274</v>
+        <v>6.95719311735195</v>
       </c>
       <c r="D119" s="208" t="n">
         <f aca="false">'Weapons Sleeve'!J54</f>
-        <v>1.15787554486341</v>
+        <v>1.14993493615936</v>
       </c>
       <c r="E119" s="209" t="n">
         <f aca="false">'Weapons Sleeve'!M54</f>
-        <v>6.90496072028128</v>
+        <v>6.98429360666453</v>
       </c>
       <c r="F119" s="210" t="n">
         <f aca="false">F118/'Weapons Sleeve'!B54</f>
-        <v>4.41312146092</v>
+        <v>4.47927207673558</v>
       </c>
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19767,23 +19777,23 @@
       </c>
       <c r="B120" s="203" t="n">
         <f aca="false">'Weapons Sleeve'!E54</f>
-        <v>0.187221251956986</v>
+        <v>0.189904683804596</v>
       </c>
       <c r="C120" s="203" t="n">
         <f aca="false">'Weapons Sleeve'!H54</f>
-        <v>0.315860226153021</v>
+        <v>0.319312637995968</v>
       </c>
       <c r="D120" s="203" t="n">
         <f aca="false">'Weapons Sleeve'!K54</f>
-        <v>0.0211617866038758</v>
+        <v>0.0201583997119177</v>
       </c>
       <c r="E120" s="204" t="n">
         <f aca="false">'Weapons Sleeve'!N54</f>
-        <v>0.317893066655618</v>
+        <v>0.32004557875878</v>
       </c>
       <c r="F120" s="205" t="n">
         <f aca="false">F119^(1/$C$100)-1</f>
-        <v>0.236250710960596</v>
+        <v>0.23888112043644</v>
       </c>
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19792,23 +19802,23 @@
       </c>
       <c r="B121" s="200" t="n">
         <f aca="false">B119/(1+'Holdco Summary'!$B$23)^$C$100</f>
-        <v>1.24978915691536</v>
+        <v>1.26969770842981</v>
       </c>
       <c r="C121" s="200" t="n">
         <f aca="false">C119/(1+'Holdco Summary'!$B$23)^$C$100</f>
-        <v>2.56793151356787</v>
+        <v>2.61546658671061</v>
       </c>
       <c r="D121" s="200" t="n">
         <f aca="false">D119/(1+'Holdco Summary'!$B$23)^$C$100</f>
-        <v>0.435288304935287</v>
+        <v>0.432303136003901</v>
       </c>
       <c r="E121" s="200" t="n">
         <f aca="false">E119/(1+'Holdco Summary'!$B$23)^$C$100</f>
-        <v>2.59583049396777</v>
+        <v>2.62565466444324</v>
       </c>
       <c r="F121" s="200" t="n">
         <f aca="false">F119/(1+'Holdco Summary'!$B$23)^$C$100</f>
-        <v>1.65905581883934</v>
+        <v>1.68392428553814</v>
       </c>
     </row>
   </sheetData>
@@ -20382,23 +20392,23 @@
       </c>
       <c r="B6" s="17" t="n">
         <f aca="false">'Holdco Summary'!F61</f>
-        <v>0.192180867725363</v>
+        <v>0.193673267252674</v>
       </c>
       <c r="C6" s="18" t="n">
         <f aca="false">'Holdco Summary'!F59</f>
-        <v>3.42290649540101</v>
+        <v>3.45301348617188</v>
       </c>
       <c r="D6" s="19" t="n">
         <f aca="false">'Holdco Summary'!F58</f>
-        <v>2875.24145613685</v>
+        <v>2952.32653067696</v>
       </c>
       <c r="E6" s="18" t="n">
         <f aca="false">'Holdco Summary'!F64</f>
-        <v>1.28679733581458</v>
+        <v>1.29811566880597</v>
       </c>
       <c r="F6" s="18" t="n">
         <f aca="false">'Holdco Summary'!F62</f>
-        <v>1.87244706988098</v>
+        <v>1.88891662484182</v>
       </c>
       <c r="G6" s="1"/>
     </row>
@@ -20449,23 +20459,23 @@
       </c>
       <c r="B10" s="21" t="n">
         <f aca="false">'Holdco Summary'!B40</f>
-        <v>0.155069571921647</v>
+        <v>0.156236964998106</v>
       </c>
       <c r="C10" s="21" t="n">
         <f aca="false">'Holdco Summary'!C40</f>
-        <v>0.271525962366753</v>
+        <v>0.273025081505314</v>
       </c>
       <c r="D10" s="21" t="n">
         <f aca="false">'Holdco Summary'!D40</f>
-        <v>-0.053663530570773</v>
+        <v>-0.053191710305405</v>
       </c>
       <c r="E10" s="21" t="n">
         <f aca="false">'Holdco Summary'!E40</f>
-        <v>0.211941654166605</v>
+        <v>0.214318971802798</v>
       </c>
       <c r="F10" s="17" t="n">
         <f aca="false">'Holdco Summary'!F40</f>
-        <v>0.177352715458623</v>
+        <v>0.178779502986822</v>
       </c>
       <c r="G10" s="1"/>
     </row>
@@ -20475,23 +20485,23 @@
       </c>
       <c r="B11" s="21" t="n">
         <f aca="false">'Holdco Summary'!B61</f>
-        <v>0.158995489652759</v>
+        <v>0.160229366235885</v>
       </c>
       <c r="C11" s="21" t="n">
         <f aca="false">'Holdco Summary'!C61</f>
-        <v>0.280230644478965</v>
+        <v>0.281797106824369</v>
       </c>
       <c r="D11" s="21" t="n">
         <f aca="false">'Holdco Summary'!D61</f>
-        <v>-0.0507794883216116</v>
+        <v>-0.0504059739765521</v>
       </c>
       <c r="E11" s="21" t="n">
         <f aca="false">'Holdco Summary'!E61</f>
-        <v>0.231808313482553</v>
+        <v>0.234046609741583</v>
       </c>
       <c r="F11" s="17" t="n">
         <f aca="false">'Holdco Summary'!F61</f>
-        <v>0.192180867725363</v>
+        <v>0.193673267252674</v>
       </c>
       <c r="G11" s="1"/>
     </row>
@@ -20501,23 +20511,23 @@
       </c>
       <c r="B12" s="21" t="n">
         <f aca="false">'Holdco Summary'!B82</f>
-        <v>0.164649431844847</v>
+        <v>0.165952502895083</v>
       </c>
       <c r="C12" s="21" t="n">
         <f aca="false">'Holdco Summary'!C82</f>
-        <v>0.291284942436493</v>
+        <v>0.292894592849268</v>
       </c>
       <c r="D12" s="21" t="n">
         <f aca="false">'Holdco Summary'!D82</f>
-        <v>-0.0462072190141125</v>
+        <v>-0.045985312895805</v>
       </c>
       <c r="E12" s="21" t="n">
         <f aca="false">'Holdco Summary'!E82</f>
-        <v>0.25472957508494</v>
+        <v>0.256733550220737</v>
       </c>
       <c r="F12" s="17" t="n">
         <f aca="false">'Holdco Summary'!F82</f>
-        <v>0.211877816332995</v>
+        <v>0.213415331908954</v>
       </c>
       <c r="G12" s="1"/>
     </row>
@@ -20568,23 +20578,23 @@
       </c>
       <c r="B16" s="22" t="n">
         <f aca="false">'Holdco Summary'!B38</f>
-        <v>2.05608335266037</v>
+        <v>2.06649447492898</v>
       </c>
       <c r="C16" s="22" t="n">
         <f aca="false">'Holdco Summary'!C38</f>
-        <v>3.32373324250012</v>
+        <v>3.3433727747867</v>
       </c>
       <c r="D16" s="22" t="n">
         <f aca="false">'Holdco Summary'!D38</f>
-        <v>0.758975724072158</v>
+        <v>0.760869645511103</v>
       </c>
       <c r="E16" s="22" t="n">
         <f aca="false">'Holdco Summary'!E38</f>
-        <v>2.61461989630139</v>
+        <v>2.64036459832027</v>
       </c>
       <c r="F16" s="18" t="n">
         <f aca="false">'Holdco Summary'!F38</f>
-        <v>2.26221016237823</v>
+        <v>2.27595084398942</v>
       </c>
       <c r="G16" s="1"/>
     </row>
@@ -20594,23 +20604,23 @@
       </c>
       <c r="B17" s="22" t="n">
         <f aca="false">'Holdco Summary'!B59</f>
-        <v>2.80913247902411</v>
+        <v>2.83013384503586</v>
       </c>
       <c r="C17" s="22" t="n">
         <f aca="false">'Holdco Summary'!C59</f>
-        <v>5.63660406983273</v>
+        <v>5.68505942879856</v>
       </c>
       <c r="D17" s="22" t="n">
         <f aca="false">'Holdco Summary'!D59</f>
-        <v>0.694336186963116</v>
+        <v>0.696250975084011</v>
       </c>
       <c r="E17" s="22" t="n">
         <f aca="false">'Holdco Summary'!E59</f>
-        <v>4.30330289558338</v>
+        <v>4.35833834962331</v>
       </c>
       <c r="F17" s="18" t="n">
         <f aca="false">'Holdco Summary'!F59</f>
-        <v>3.42290649540101</v>
+        <v>3.45301348617188</v>
       </c>
       <c r="G17" s="1"/>
     </row>
@@ -20620,23 +20630,23 @@
       </c>
       <c r="B18" s="22" t="n">
         <f aca="false">'Holdco Summary'!B80</f>
-        <v>4.59147465749586</v>
+        <v>4.64310591330418</v>
       </c>
       <c r="C18" s="22" t="n">
         <f aca="false">'Holdco Summary'!C80</f>
-        <v>12.8890487954669</v>
+        <v>13.0506214172789</v>
       </c>
       <c r="D18" s="22" t="n">
         <f aca="false">'Holdco Summary'!D80</f>
-        <v>0.623074977486035</v>
+        <v>0.62452612073781</v>
       </c>
       <c r="E18" s="22" t="n">
         <f aca="false">'Holdco Summary'!E80</f>
-        <v>9.67166729025792</v>
+        <v>9.82725200925749</v>
       </c>
       <c r="F18" s="18" t="n">
         <f aca="false">'Holdco Summary'!F80</f>
-        <v>6.83263713490145</v>
+        <v>6.9198197348059</v>
       </c>
       <c r="G18" s="1"/>
     </row>
@@ -20687,23 +20697,23 @@
       </c>
       <c r="B22" s="23" t="n">
         <f aca="false">'Holdco Summary'!B37</f>
-        <v>1727.11001623471</v>
+        <v>1766.85277606428</v>
       </c>
       <c r="C22" s="23" t="n">
         <f aca="false">'Holdco Summary'!C37</f>
-        <v>2791.9359237001</v>
+        <v>2858.58372244263</v>
       </c>
       <c r="D22" s="23" t="n">
         <f aca="false">'Holdco Summary'!D37</f>
-        <v>637.539608220613</v>
+        <v>650.543546911993</v>
       </c>
       <c r="E22" s="23" t="n">
         <f aca="false">'Holdco Summary'!E37</f>
-        <v>2196.28071289317</v>
+        <v>2257.51173156383</v>
       </c>
       <c r="F22" s="19" t="n">
         <f aca="false">'Holdco Summary'!F37</f>
-        <v>1900.25653639771</v>
+        <v>1945.93797161096</v>
       </c>
       <c r="G22" s="1"/>
     </row>
@@ -20713,23 +20723,23 @@
       </c>
       <c r="B23" s="23" t="n">
         <f aca="false">'Holdco Summary'!B58</f>
-        <v>2359.67128238025</v>
+        <v>2419.76443750566</v>
       </c>
       <c r="C23" s="23" t="n">
         <f aca="false">'Holdco Summary'!C58</f>
-        <v>4734.74741865949</v>
+        <v>4860.72581162277</v>
       </c>
       <c r="D23" s="23" t="n">
         <f aca="false">'Holdco Summary'!D58</f>
-        <v>583.242397049017</v>
+        <v>595.29458369683</v>
       </c>
       <c r="E23" s="23" t="n">
         <f aca="false">'Holdco Summary'!E58</f>
-        <v>3614.77443229004</v>
+        <v>3726.37928892793</v>
       </c>
       <c r="F23" s="19" t="n">
         <f aca="false">'Holdco Summary'!F58</f>
-        <v>2875.24145613685</v>
+        <v>2952.32653067696</v>
       </c>
       <c r="G23" s="1"/>
     </row>
@@ -20739,23 +20749,23 @@
       </c>
       <c r="B24" s="23" t="n">
         <f aca="false">'Holdco Summary'!B79</f>
-        <v>3856.83871229652</v>
+        <v>3969.85555587508</v>
       </c>
       <c r="C24" s="23" t="n">
         <f aca="false">'Holdco Summary'!C79</f>
-        <v>10826.8009881922</v>
+        <v>11158.2813117735</v>
       </c>
       <c r="D24" s="23" t="n">
         <f aca="false">'Holdco Summary'!D79</f>
-        <v>523.38298108827</v>
+        <v>533.969833230827</v>
       </c>
       <c r="E24" s="23" t="n">
         <f aca="false">'Holdco Summary'!E79</f>
-        <v>8124.20052381665</v>
+        <v>8402.30046791515</v>
       </c>
       <c r="F24" s="19" t="n">
         <f aca="false">'Holdco Summary'!F79</f>
-        <v>5739.41519331722</v>
+        <v>5916.44587325905</v>
       </c>
       <c r="G24" s="1"/>
     </row>
@@ -20806,23 +20816,23 @@
       </c>
       <c r="B28" s="22" t="n">
         <f aca="false">'Holdco Summary'!B43</f>
-        <v>1.02223680877684</v>
+        <v>1.02741297655714</v>
       </c>
       <c r="C28" s="22" t="n">
         <f aca="false">'Holdco Summary'!C43</f>
-        <v>1.65248284250861</v>
+        <v>1.66224716105364</v>
       </c>
       <c r="D28" s="22" t="n">
         <f aca="false">'Holdco Summary'!D43</f>
-        <v>0.377345072664851</v>
+        <v>0.378286686342777</v>
       </c>
       <c r="E28" s="22" t="n">
         <f aca="false">'Holdco Summary'!E43</f>
-        <v>1.29992818408908</v>
+        <v>1.31272785099005</v>
       </c>
       <c r="F28" s="18" t="n">
         <f aca="false">'Holdco Summary'!F43</f>
-        <v>1.12471826308982</v>
+        <v>1.13154981031405</v>
       </c>
       <c r="G28" s="1"/>
     </row>
@@ -20832,23 +20842,23 @@
       </c>
       <c r="B29" s="22" t="n">
         <f aca="false">'Holdco Summary'!B64</f>
-        <v>1.05605694891614</v>
+        <v>1.06395214028894</v>
       </c>
       <c r="C29" s="22" t="n">
         <f aca="false">'Holdco Summary'!C64</f>
-        <v>2.11900824923137</v>
+        <v>2.1372244134494</v>
       </c>
       <c r="D29" s="22" t="n">
         <f aca="false">'Holdco Summary'!D64</f>
-        <v>0.261026690838401</v>
+        <v>0.26174653061665</v>
       </c>
       <c r="E29" s="22" t="n">
         <f aca="false">'Holdco Summary'!E64</f>
-        <v>1.61777095245809</v>
+        <v>1.63846081814068</v>
       </c>
       <c r="F29" s="18" t="n">
         <f aca="false">'Holdco Summary'!F64</f>
-        <v>1.28679733581458</v>
+        <v>1.29811566880597</v>
       </c>
       <c r="G29" s="1"/>
     </row>
@@ -20858,23 +20868,23 @@
       </c>
       <c r="B30" s="22" t="n">
         <f aca="false">'Holdco Summary'!B85</f>
-        <v>1.13494231387911</v>
+        <v>1.14770477067279</v>
       </c>
       <c r="C30" s="22" t="n">
         <f aca="false">'Holdco Summary'!C85</f>
-        <v>3.18597573869788</v>
+        <v>3.22591401973781</v>
       </c>
       <c r="D30" s="22" t="n">
         <f aca="false">'Holdco Summary'!D85</f>
-        <v>0.154014605201774</v>
+        <v>0.154373305620004</v>
       </c>
       <c r="E30" s="22" t="n">
         <f aca="false">'Holdco Summary'!E85</f>
-        <v>2.39068823685087</v>
+        <v>2.42914639989383</v>
       </c>
       <c r="F30" s="18" t="n">
         <f aca="false">'Holdco Summary'!F85</f>
-        <v>1.68892340222796</v>
+        <v>1.71047360756428</v>
       </c>
       <c r="G30" s="1"/>
     </row>
@@ -20925,23 +20935,23 @@
       </c>
       <c r="B34" s="22" t="n">
         <f aca="false">'Holdco Summary'!B41</f>
-        <v>1.3363131037395</v>
+        <v>1.34307961886846</v>
       </c>
       <c r="C34" s="22" t="n">
         <f aca="false">'Holdco Summary'!C41</f>
-        <v>2.160198553984</v>
+        <v>2.17296290242927</v>
       </c>
       <c r="D34" s="22" t="n">
         <f aca="false">'Holdco Summary'!D41</f>
-        <v>0.493282144513008</v>
+        <v>0.494513063499362</v>
       </c>
       <c r="E34" s="22" t="n">
         <f aca="false">'Holdco Summary'!E41</f>
-        <v>1.6993235338464</v>
+        <v>1.71605582371937</v>
       </c>
       <c r="F34" s="18" t="n">
         <f aca="false">'Holdco Summary'!F41</f>
-        <v>1.47028138693269</v>
+        <v>1.47921188718093</v>
       </c>
       <c r="G34" s="1"/>
     </row>
@@ -20951,23 +20961,23 @@
       </c>
       <c r="B35" s="22" t="n">
         <f aca="false">'Holdco Summary'!B62</f>
-        <v>1.53669166432779</v>
+        <v>1.54818013072471</v>
       </c>
       <c r="C35" s="22" t="n">
         <f aca="false">'Holdco Summary'!C62</f>
-        <v>3.08341545082172</v>
+        <v>3.1099221915222</v>
       </c>
       <c r="D35" s="22" t="n">
         <f aca="false">'Holdco Summary'!D62</f>
-        <v>0.379825671702756</v>
+        <v>0.380873126376505</v>
       </c>
       <c r="E35" s="22" t="n">
         <f aca="false">'Holdco Summary'!E62</f>
-        <v>2.35405404981752</v>
+        <v>2.38416032785786</v>
       </c>
       <c r="F35" s="18" t="n">
         <f aca="false">'Holdco Summary'!F62</f>
-        <v>1.87244706988098</v>
+        <v>1.88891662484182</v>
       </c>
       <c r="G35" s="1"/>
     </row>
@@ -20977,23 +20987,23 @@
       </c>
       <c r="B36" s="22" t="n">
         <f aca="false">'Holdco Summary'!B83</f>
-        <v>1.93948851491393</v>
+        <v>1.96129811534096</v>
       </c>
       <c r="C36" s="22" t="n">
         <f aca="false">'Holdco Summary'!C83</f>
-        <v>5.44447350181108</v>
+        <v>5.51272352336294</v>
       </c>
       <c r="D36" s="22" t="n">
         <f aca="false">'Holdco Summary'!D83</f>
-        <v>0.263193603996389</v>
+        <v>0.263806582588293</v>
       </c>
       <c r="E36" s="22" t="n">
         <f aca="false">'Holdco Summary'!E83</f>
-        <v>4.08541678410449</v>
+        <v>4.15113745079773</v>
       </c>
       <c r="F36" s="18" t="n">
         <f aca="false">'Holdco Summary'!F83</f>
-        <v>2.88617976537917</v>
+        <v>2.92300663775207</v>
       </c>
       <c r="G36" s="1"/>
     </row>
@@ -21045,7 +21055,7 @@
       </c>
       <c r="C40" s="21" t="n">
         <f aca="false">'Holdco Summary'!C6</f>
-        <v>0.297619047619048</v>
+        <v>0.292397660818713</v>
       </c>
       <c r="D40" s="26" t="n">
         <f aca="false">COUNT(Assumptions!C18:C26)</f>
@@ -21062,11 +21072,11 @@
       </c>
       <c r="B41" s="25" t="n">
         <f aca="false">'Holdco Summary'!B7</f>
-        <v>390</v>
+        <v>405</v>
       </c>
       <c r="C41" s="21" t="n">
         <f aca="false">'Holdco Summary'!C7</f>
-        <v>0.464285714285714</v>
+        <v>0.473684210526316</v>
       </c>
       <c r="D41" s="26" t="n">
         <f aca="false">COUNT('Weapons Sleeve'!C12:C22)</f>
@@ -21087,7 +21097,7 @@
       </c>
       <c r="C42" s="21" t="n">
         <f aca="false">'Holdco Summary'!C8</f>
-        <v>0.238095238095238</v>
+        <v>0.233918128654971</v>
       </c>
       <c r="D42" s="26" t="n">
         <f aca="false">COUNT('Consumer Sleeve'!C12:C20)</f>
@@ -21103,7 +21113,7 @@
       </c>
       <c r="B43" s="28" t="n">
         <f aca="false">SUM(B40:B42)</f>
-        <v>840</v>
+        <v>855</v>
       </c>
       <c r="C43" s="29" t="n">
         <f aca="false">SUM(C40:C42)</f>
@@ -21190,23 +21200,23 @@
       </c>
       <c r="B48" s="31" t="n">
         <f aca="false">'Holdco Summary'!B29/'Holdco Summary'!$B$7</f>
-        <v>2.34791206742085</v>
+        <v>2.37463994022986</v>
       </c>
       <c r="C48" s="31" t="n">
         <f aca="false">'Holdco Summary'!C29/'Holdco Summary'!$B$7</f>
-        <v>3.89233680586787</v>
+        <v>3.94490400599662</v>
       </c>
       <c r="D48" s="31" t="n">
         <f aca="false">'Holdco Summary'!D29/'Holdco Summary'!$B$7</f>
-        <v>1.11273632367401</v>
+        <v>1.10733606154135</v>
       </c>
       <c r="E48" s="31" t="n">
         <f aca="false">'Holdco Summary'!E29/'Holdco Summary'!$B$7</f>
-        <v>3.92700209637202</v>
+        <v>3.96156693984054</v>
       </c>
       <c r="F48" s="31" t="n">
         <f aca="false">'Holdco Summary'!F29/'Holdco Summary'!$B$7</f>
-        <v>2.78560539481325</v>
+        <v>2.81514942480987</v>
       </c>
       <c r="G48" s="1"/>
     </row>
@@ -21242,23 +21252,23 @@
       </c>
       <c r="B50" s="32" t="n">
         <f aca="false">'Holdco Summary'!B31/'Holdco Summary'!$B$9</f>
-        <v>2.32777217162546</v>
+        <v>2.34078607446123</v>
       </c>
       <c r="C50" s="32" t="n">
         <f aca="false">'Holdco Summary'!C31/'Holdco Summary'!$B$9</f>
-        <v>3.91233453392515</v>
+        <v>3.93688394928338</v>
       </c>
       <c r="D50" s="32" t="n">
         <f aca="false">'Holdco Summary'!D31/'Holdco Summary'!$B$9</f>
-        <v>0.858975724072158</v>
+        <v>0.860869645511103</v>
       </c>
       <c r="E50" s="32" t="n">
         <f aca="false">'Holdco Summary'!E31/'Holdco Summary'!$B$9</f>
-        <v>3.02594285117673</v>
+        <v>3.05812372870034</v>
       </c>
       <c r="F50" s="32" t="n">
         <f aca="false">'Holdco Summary'!F31/'Holdco Summary'!$B$9</f>
-        <v>2.60831889700008</v>
+        <v>2.62542372696011</v>
       </c>
       <c r="G50" s="1"/>
     </row>
@@ -21335,23 +21345,23 @@
       </c>
       <c r="B55" s="31" t="n">
         <f aca="false">'Holdco Summary'!B50/'Holdco Summary'!$B$7</f>
-        <v>3.32446400378914</v>
+        <v>3.3774211466089</v>
       </c>
       <c r="C55" s="31" t="n">
         <f aca="false">'Holdco Summary'!C50/'Holdco Summary'!$B$7</f>
-        <v>6.83074887777274</v>
+        <v>6.95719311735195</v>
       </c>
       <c r="D55" s="31" t="n">
         <f aca="false">'Holdco Summary'!D50/'Holdco Summary'!$B$7</f>
-        <v>1.15787554486341</v>
+        <v>1.14993493615936</v>
       </c>
       <c r="E55" s="31" t="n">
         <f aca="false">'Holdco Summary'!E50/'Holdco Summary'!$B$7</f>
-        <v>6.90496072028128</v>
+        <v>6.98429360666453</v>
       </c>
       <c r="F55" s="31" t="n">
         <f aca="false">'Holdco Summary'!F50/'Holdco Summary'!$B$7</f>
-        <v>4.41312146092</v>
+        <v>4.47927207673558</v>
       </c>
       <c r="G55" s="1"/>
     </row>
@@ -21387,23 +21397,23 @@
       </c>
       <c r="B57" s="32" t="n">
         <f aca="false">'Holdco Summary'!B52/'Holdco Summary'!$B$9</f>
-        <v>3.25795953158525</v>
+        <v>3.28421123909995</v>
       </c>
       <c r="C57" s="32" t="n">
         <f aca="false">'Holdco Summary'!C52/'Holdco Summary'!$B$9</f>
-        <v>6.79229902009603</v>
+        <v>6.85286821880332</v>
       </c>
       <c r="D57" s="32" t="n">
         <f aca="false">'Holdco Summary'!D52/'Holdco Summary'!$B$9</f>
-        <v>0.834336186963116</v>
+        <v>0.836250975084011</v>
       </c>
       <c r="E57" s="32" t="n">
         <f aca="false">'Holdco Summary'!E52/'Holdco Summary'!$B$9</f>
-        <v>5.12567255228435</v>
+        <v>5.19446686983425</v>
       </c>
       <c r="F57" s="32" t="n">
         <f aca="false">'Holdco Summary'!F52/'Holdco Summary'!$B$9</f>
-        <v>4.05815785512449</v>
+        <v>4.09571978903355</v>
       </c>
       <c r="G57" s="1"/>
     </row>
@@ -21480,23 +21490,23 @@
       </c>
       <c r="B62" s="31" t="n">
         <f aca="false">'Holdco Summary'!B71/'Holdco Summary'!$B$7</f>
-        <v>5.68435978733779</v>
+        <v>5.81191457480287</v>
       </c>
       <c r="C62" s="31" t="n">
         <f aca="false">'Holdco Summary'!C71/'Holdco Summary'!$B$7</f>
-        <v>16.3149383848512</v>
+        <v>16.7230380390834</v>
       </c>
       <c r="D62" s="31" t="n">
         <f aca="false">'Holdco Summary'!D71/'Holdco Summary'!$B$7</f>
-        <v>1.2332898185244</v>
+        <v>1.22116020090635</v>
       </c>
       <c r="E62" s="31" t="n">
         <f aca="false">'Holdco Summary'!E71/'Holdco Summary'!$B$7</f>
-        <v>16.534742164625</v>
+        <v>16.7699466804619</v>
       </c>
       <c r="F62" s="31" t="n">
         <f aca="false">'Holdco Summary'!F71/'Holdco Summary'!$B$7</f>
-        <v>9.30190129798722</v>
+        <v>9.49478710063738</v>
       </c>
       <c r="G62" s="1"/>
     </row>
@@ -21532,23 +21542,23 @@
       </c>
       <c r="B64" s="32" t="n">
         <f aca="false">'Holdco Summary'!B73/'Holdco Summary'!$B$9</f>
-        <v>5.44961207255162</v>
+        <v>5.51415114231203</v>
       </c>
       <c r="C64" s="32" t="n">
         <f aca="false">'Holdco Summary'!C73/'Holdco Summary'!$B$9</f>
-        <v>15.8215797450154</v>
+        <v>16.0235455222804</v>
       </c>
       <c r="D64" s="32" t="n">
         <f aca="false">'Holdco Summary'!D73/'Holdco Summary'!$B$9</f>
-        <v>0.823074977486035</v>
+        <v>0.82452612073781</v>
       </c>
       <c r="E64" s="32" t="n">
         <f aca="false">'Holdco Summary'!E73/'Holdco Summary'!$B$9</f>
-        <v>11.7998528635042</v>
+        <v>11.9943337622537</v>
       </c>
       <c r="F64" s="32" t="n">
         <f aca="false">'Holdco Summary'!F73/'Holdco Summary'!$B$9</f>
-        <v>8.30115954505063</v>
+        <v>8.41008337705924</v>
       </c>
       <c r="G64" s="1"/>
     </row>
@@ -21660,10 +21670,10 @@
       </c>
       <c r="B72" s="34" t="n">
         <f aca="false">'Holdco Summary'!B9</f>
-        <v>840</v>
+        <v>855</v>
       </c>
       <c r="C72" s="35" t="n">
-        <v>840</v>
+        <v>855</v>
       </c>
       <c r="D72" s="36" t="str">
         <f aca="false">IF(ABS(B72-C72)&lt;0.001,"OK","CHECK")</f>
@@ -21699,11 +21709,11 @@
       </c>
       <c r="B74" s="34" t="n">
         <f aca="false">'Weapons Sleeve'!C23</f>
-        <v>390</v>
+        <v>405</v>
       </c>
       <c r="C74" s="34" t="n">
         <f aca="false">'Weapons Sleeve'!B5</f>
-        <v>390</v>
+        <v>405</v>
       </c>
       <c r="D74" s="36" t="str">
         <f aca="false">IF(ABS(B74-C74)&lt;0.001,"OK","CHECK")</f>
@@ -21796,11 +21806,11 @@
       </c>
       <c r="B79" s="34" t="n">
         <f aca="false">'Holdco Summary'!F52</f>
-        <v>3408.85259830457</v>
+        <v>3501.84041962368</v>
       </c>
       <c r="C79" s="34" t="n">
         <f aca="false">'Fund Economics'!F22+'Holdco Summary'!F50+'Holdco Summary'!F51</f>
-        <v>3408.85259830457</v>
+        <v>3501.84041962368</v>
       </c>
       <c r="D79" s="36" t="str">
         <f aca="false">IF(ABS(B79-C79)&lt;0.001,"OK","CHECK")</f>
@@ -21847,7 +21857,7 @@
     <row r="83" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A83" s="40" t="str">
         <f aca="false">"• Underwrite to Expected: 7-yr holdco net IRR "&amp;TEXT('Holdco Summary'!F61,"0.0%")&amp;" / "&amp;TEXT('Holdco Summary'!F59,"0.00")&amp;"x net MOIC; Base "&amp;TEXT('Holdco Summary'!B61,"0.0%")&amp;", Bear "&amp;TEXT('Holdco Summary'!D61,"0.0%")&amp;"."</f>
-        <v>• Underwrite to Expected: 7-yr holdco net IRR 19.2% / 3.42x net MOIC; Base 15.9%, Bear -5.1%.</v>
+        <v>• Underwrite to Expected: 7-yr holdco net IRR 19.4% / 3.45x net MOIC; Base 16.0%, Bear -5.0%.</v>
       </c>
       <c r="B83" s="40"/>
       <c r="C83" s="40"/>
@@ -21859,7 +21869,7 @@
     <row r="84" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A84" s="40" t="str">
         <f aca="false">"• Thematic scoreboard: 7-yr Expected KS-PME vs Defense+Semis basket "&amp;TEXT('Holdco Summary'!F64,"0.00")&amp;"x (Base "&amp;TEXT('Holdco Summary'!B64,"0.00")&amp;"x) — &gt;1.00x means the holdco beats owning ITA/SOXX."</f>
-        <v>• Thematic scoreboard: 7-yr Expected KS-PME vs Defense+Semis basket 1.29x (Base 1.06x) — &gt;1.00x means the holdco beats owning ITA/SOXX.</v>
+        <v>• Thematic scoreboard: 7-yr Expected KS-PME vs Defense+Semis basket 1.30x (Base 1.06x) — &gt;1.00x means the holdco beats owning ITA/SOXX.</v>
       </c>
       <c r="B84" s="40"/>
       <c r="C84" s="40"/>
@@ -22005,7 +22015,7 @@
       </c>
       <c r="C6" s="46" t="n">
         <f aca="false">B6/$B$9</f>
-        <v>0.297619047619048</v>
+        <v>0.292397660818713</v>
       </c>
       <c r="D6" s="47" t="s">
         <v>89</v>
@@ -22022,11 +22032,11 @@
         <v>92</v>
       </c>
       <c r="B7" s="49" t="n">
-        <v>390</v>
+        <v>405</v>
       </c>
       <c r="C7" s="46" t="n">
         <f aca="false">B7/$B$9</f>
-        <v>0.464285714285714</v>
+        <v>0.473684210526316</v>
       </c>
       <c r="D7" s="47" t="s">
         <v>93</v>
@@ -22047,7 +22057,7 @@
       </c>
       <c r="C8" s="46" t="n">
         <f aca="false">B8/$B$9</f>
-        <v>0.238095238095238</v>
+        <v>0.233918128654971</v>
       </c>
       <c r="D8" s="47" t="s">
         <v>96</v>
@@ -22065,7 +22075,7 @@
       </c>
       <c r="B9" s="50" t="n">
         <f aca="false">SUM(B6:B8)</f>
-        <v>840</v>
+        <v>855</v>
       </c>
       <c r="C9" s="51" t="n">
         <f aca="false">SUM(C6:C8)</f>
@@ -22322,23 +22332,23 @@
       </c>
       <c r="B29" s="62" t="n">
         <f aca="false">'Weapons Sleeve'!C38</f>
-        <v>915.68570629413</v>
+        <v>961.729175793093</v>
       </c>
       <c r="C29" s="62" t="n">
         <f aca="false">'Weapons Sleeve'!F38</f>
-        <v>1518.01135428847</v>
+        <v>1597.68612242863</v>
       </c>
       <c r="D29" s="62" t="n">
         <f aca="false">'Weapons Sleeve'!I38</f>
-        <v>433.967166232866</v>
+        <v>448.471104924246</v>
       </c>
       <c r="E29" s="63" t="n">
         <f aca="false">'Weapons Sleeve'!L38</f>
-        <v>1531.53081758509</v>
+        <v>1604.43461063542</v>
       </c>
       <c r="F29" s="64" t="n">
         <f aca="false">B29*'Defense Supercycle'!$B$17+C29*'Defense Supercycle'!$B$18+D29*'Defense Supercycle'!$B$19+E29*'Defense Supercycle'!$B$20</f>
-        <v>1086.38610397717</v>
+        <v>1140.135517048</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22372,23 +22382,23 @@
       </c>
       <c r="B31" s="66" t="n">
         <f aca="false">B28+B29+B30</f>
-        <v>1955.32862416539</v>
+        <v>2001.37209366435</v>
       </c>
       <c r="C31" s="66" t="n">
         <f aca="false">C28+C29+C30</f>
-        <v>3286.36100849713</v>
+        <v>3366.03577663729</v>
       </c>
       <c r="D31" s="66" t="n">
         <f aca="false">D28+D29+D30</f>
-        <v>721.539608220613</v>
+        <v>736.043546911993</v>
       </c>
       <c r="E31" s="66" t="n">
         <f aca="false">E28+E29+E30</f>
-        <v>2541.79199498846</v>
+        <v>2614.69578803879</v>
       </c>
       <c r="F31" s="66" t="n">
         <f aca="false">F28+F29+F30</f>
-        <v>2190.98787348007</v>
+        <v>2244.7372865509</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22397,23 +22407,23 @@
       </c>
       <c r="B32" s="62" t="n">
         <f aca="false">-'Holdco Summary'!$B$9</f>
-        <v>-840</v>
+        <v>-855</v>
       </c>
       <c r="C32" s="62" t="n">
         <f aca="false">-'Holdco Summary'!$B$9</f>
-        <v>-840</v>
+        <v>-855</v>
       </c>
       <c r="D32" s="62" t="n">
         <f aca="false">-'Holdco Summary'!$B$9</f>
-        <v>-840</v>
+        <v>-855</v>
       </c>
       <c r="E32" s="63" t="n">
         <f aca="false">-'Holdco Summary'!$B$9</f>
-        <v>-840</v>
+        <v>-855</v>
       </c>
       <c r="F32" s="64" t="n">
         <f aca="false">-'Holdco Summary'!$B$9</f>
-        <v>-840</v>
+        <v>-855</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22422,23 +22432,23 @@
       </c>
       <c r="B33" s="62" t="n">
         <f aca="false">-'Holdco Summary'!$B$9*((1+Assumptions!$B$10)^5-1)</f>
-        <v>-394.235584512</v>
+        <v>-401.275505664001</v>
       </c>
       <c r="C33" s="62" t="n">
         <f aca="false">-'Holdco Summary'!$B$9*((1+Assumptions!$B$10)^5-1)</f>
-        <v>-394.235584512</v>
+        <v>-401.275505664001</v>
       </c>
       <c r="D33" s="62" t="n">
         <f aca="false">-'Holdco Summary'!$B$9*((1+Assumptions!$B$10)^5-1)</f>
-        <v>-394.235584512</v>
+        <v>-401.275505664001</v>
       </c>
       <c r="E33" s="63" t="n">
         <f aca="false">-'Holdco Summary'!$B$9*((1+Assumptions!$B$10)^5-1)</f>
-        <v>-394.235584512</v>
+        <v>-401.275505664001</v>
       </c>
       <c r="F33" s="64" t="n">
         <f aca="false">-'Holdco Summary'!$B$9*((1+Assumptions!$B$10)^5-1)</f>
-        <v>-394.235584512</v>
+        <v>-401.275505664001</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22447,11 +22457,11 @@
       </c>
       <c r="B34" s="62" t="n">
         <f aca="false">MAX(0,B31+B32+B33)</f>
-        <v>721.093039653385</v>
+        <v>745.096588000347</v>
       </c>
       <c r="C34" s="62" t="n">
         <f aca="false">MAX(0,C31+C32+C33)</f>
-        <v>2052.12542398512</v>
+        <v>2109.76027097329</v>
       </c>
       <c r="D34" s="62" t="n">
         <f aca="false">MAX(0,D31+D32+D33)</f>
@@ -22459,11 +22469,11 @@
       </c>
       <c r="E34" s="63" t="n">
         <f aca="false">MAX(0,E31+E32+E33)</f>
-        <v>1307.55641047646</v>
+        <v>1358.42028237479</v>
       </c>
       <c r="F34" s="64" t="n">
         <f aca="false">B34*'Defense Supercycle'!$B$17+C34*'Defense Supercycle'!$B$18+D34*'Defense Supercycle'!$B$19+E34*'Defense Supercycle'!$B$20</f>
-        <v>1033.65668541177</v>
+        <v>1066.4965746997</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22472,11 +22482,11 @@
       </c>
       <c r="B35" s="62" t="n">
         <f aca="false">-Assumptions!$B$9*B34</f>
-        <v>-144.218607930677</v>
+        <v>-149.019317600069</v>
       </c>
       <c r="C35" s="62" t="n">
         <f aca="false">-Assumptions!$B$9*C34</f>
-        <v>-410.425084797025</v>
+        <v>-421.952054194657</v>
       </c>
       <c r="D35" s="62" t="n">
         <f aca="false">-Assumptions!$B$9*D34</f>
@@ -22484,11 +22494,11 @@
       </c>
       <c r="E35" s="63" t="n">
         <f aca="false">-Assumptions!$B$9*E34</f>
-        <v>-261.511282095291</v>
+        <v>-271.684056474957</v>
       </c>
       <c r="F35" s="64" t="n">
         <f aca="false">B35*'Defense Supercycle'!$B$17+C35*'Defense Supercycle'!$B$18+D35*'Defense Supercycle'!$B$19+E35*'Defense Supercycle'!$B$20</f>
-        <v>-206.731337082355</v>
+        <v>-213.299314939939</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22497,23 +22507,23 @@
       </c>
       <c r="B36" s="62" t="n">
         <f aca="false">-'Holdco Summary'!$B$9*Assumptions!$B$8*5</f>
-        <v>-84</v>
+        <v>-85.5</v>
       </c>
       <c r="C36" s="62" t="n">
         <f aca="false">-'Holdco Summary'!$B$9*Assumptions!$B$8*5</f>
-        <v>-84</v>
+        <v>-85.5</v>
       </c>
       <c r="D36" s="62" t="n">
         <f aca="false">-'Holdco Summary'!$B$9*Assumptions!$B$8*5</f>
-        <v>-84</v>
+        <v>-85.5</v>
       </c>
       <c r="E36" s="63" t="n">
         <f aca="false">-'Holdco Summary'!$B$9*Assumptions!$B$8*5</f>
-        <v>-84</v>
+        <v>-85.5</v>
       </c>
       <c r="F36" s="64" t="n">
         <f aca="false">-'Holdco Summary'!$B$9*Assumptions!$B$8*5</f>
-        <v>-84</v>
+        <v>-85.5</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22522,23 +22532,23 @@
       </c>
       <c r="B37" s="66" t="n">
         <f aca="false">B31+B35+B36</f>
-        <v>1727.11001623471</v>
+        <v>1766.85277606428</v>
       </c>
       <c r="C37" s="66" t="n">
         <f aca="false">C31+C35+C36</f>
-        <v>2791.9359237001</v>
+        <v>2858.58372244263</v>
       </c>
       <c r="D37" s="66" t="n">
         <f aca="false">D31+D35+D36</f>
-        <v>637.539608220613</v>
+        <v>650.543546911993</v>
       </c>
       <c r="E37" s="66" t="n">
         <f aca="false">E31+E35+E36</f>
-        <v>2196.28071289317</v>
+        <v>2257.51173156383</v>
       </c>
       <c r="F37" s="66" t="n">
         <f aca="false">F31+F35+F36</f>
-        <v>1900.25653639771</v>
+        <v>1945.93797161096</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22547,23 +22557,23 @@
       </c>
       <c r="B38" s="67" t="n">
         <f aca="false">B37/'Holdco Summary'!$B$9</f>
-        <v>2.05608335266037</v>
+        <v>2.06649447492898</v>
       </c>
       <c r="C38" s="67" t="n">
         <f aca="false">C37/'Holdco Summary'!$B$9</f>
-        <v>3.32373324250012</v>
+        <v>3.3433727747867</v>
       </c>
       <c r="D38" s="67" t="n">
         <f aca="false">D37/'Holdco Summary'!$B$9</f>
-        <v>0.758975724072158</v>
+        <v>0.760869645511103</v>
       </c>
       <c r="E38" s="67" t="n">
         <f aca="false">E37/'Holdco Summary'!$B$9</f>
-        <v>2.61461989630139</v>
+        <v>2.64036459832027</v>
       </c>
       <c r="F38" s="67" t="n">
         <f aca="false">F37/'Holdco Summary'!$B$9</f>
-        <v>2.26221016237823</v>
+        <v>2.27595084398942</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22572,23 +22582,23 @@
       </c>
       <c r="B39" s="68" t="n">
         <f aca="false">B37/'Holdco Summary'!$B$9</f>
-        <v>2.05608335266037</v>
+        <v>2.06649447492898</v>
       </c>
       <c r="C39" s="68" t="n">
         <f aca="false">C37/'Holdco Summary'!$B$9</f>
-        <v>3.32373324250012</v>
+        <v>3.3433727747867</v>
       </c>
       <c r="D39" s="68" t="n">
         <f aca="false">D37/'Holdco Summary'!$B$9</f>
-        <v>0.758975724072158</v>
+        <v>0.760869645511103</v>
       </c>
       <c r="E39" s="69" t="n">
         <f aca="false">E37/'Holdco Summary'!$B$9</f>
-        <v>2.61461989630139</v>
+        <v>2.64036459832027</v>
       </c>
       <c r="F39" s="70" t="n">
         <f aca="false">F37/'Holdco Summary'!$B$9</f>
-        <v>2.26221016237823</v>
+        <v>2.27595084398942</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22597,23 +22607,23 @@
       </c>
       <c r="B40" s="51" t="n">
         <f aca="false">(B37/'Holdco Summary'!$B$9)^(1/5)-1</f>
-        <v>0.155069571921647</v>
+        <v>0.156236964998106</v>
       </c>
       <c r="C40" s="51" t="n">
         <f aca="false">(C37/'Holdco Summary'!$B$9)^(1/5)-1</f>
-        <v>0.271525962366753</v>
+        <v>0.273025081505314</v>
       </c>
       <c r="D40" s="51" t="n">
         <f aca="false">(D37/'Holdco Summary'!$B$9)^(1/5)-1</f>
-        <v>-0.053663530570773</v>
+        <v>-0.053191710305405</v>
       </c>
       <c r="E40" s="51" t="n">
         <f aca="false">(E37/'Holdco Summary'!$B$9)^(1/5)-1</f>
-        <v>0.211941654166605</v>
+        <v>0.214318971802798</v>
       </c>
       <c r="F40" s="51" t="n">
         <f aca="false">(F37/'Holdco Summary'!$B$9)^(1/5)-1</f>
-        <v>0.177352715458623</v>
+        <v>0.178779502986822</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22622,23 +22632,23 @@
       </c>
       <c r="B41" s="68" t="n">
         <f aca="false">B38/(1+'Holdco Summary'!$B$21)^5</f>
-        <v>1.3363131037395</v>
+        <v>1.34307961886846</v>
       </c>
       <c r="C41" s="68" t="n">
         <f aca="false">C38/(1+'Holdco Summary'!$B$21)^5</f>
-        <v>2.160198553984</v>
+        <v>2.17296290242927</v>
       </c>
       <c r="D41" s="68" t="n">
         <f aca="false">D38/(1+'Holdco Summary'!$B$21)^5</f>
-        <v>0.493282144513008</v>
+        <v>0.494513063499362</v>
       </c>
       <c r="E41" s="69" t="n">
         <f aca="false">E38/(1+'Holdco Summary'!$B$21)^5</f>
-        <v>1.6993235338464</v>
+        <v>1.71605582371937</v>
       </c>
       <c r="F41" s="70" t="n">
         <f aca="false">F38/(1+'Holdco Summary'!$B$21)^5</f>
-        <v>1.47028138693269</v>
+        <v>1.47921188718093</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22647,23 +22657,23 @@
       </c>
       <c r="B42" s="68" t="n">
         <f aca="false">B38/(1+'Holdco Summary'!$B$22)^5</f>
-        <v>1.11595966889947</v>
+        <v>1.12161040895567</v>
       </c>
       <c r="C42" s="68" t="n">
         <f aca="false">C38/(1+'Holdco Summary'!$B$22)^5</f>
-        <v>1.8039892419786</v>
+        <v>1.81464879326553</v>
       </c>
       <c r="D42" s="68" t="n">
         <f aca="false">D38/(1+'Holdco Summary'!$B$22)^5</f>
-        <v>0.41194161542254</v>
+        <v>0.412969560101529</v>
       </c>
       <c r="E42" s="69" t="n">
         <f aca="false">E38/(1+'Holdco Summary'!$B$22)^5</f>
-        <v>1.41911092757943</v>
+        <v>1.43308412039952</v>
       </c>
       <c r="F42" s="70" t="n">
         <f aca="false">F38/(1+'Holdco Summary'!$B$22)^5</f>
-        <v>1.22783704294971</v>
+        <v>1.23529493442159</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22672,23 +22682,23 @@
       </c>
       <c r="B43" s="67" t="n">
         <f aca="false">B38/(1+'Holdco Summary'!$B$23)^5</f>
-        <v>1.02223680877684</v>
+        <v>1.02741297655714</v>
       </c>
       <c r="C43" s="67" t="n">
         <f aca="false">C38/(1+'Holdco Summary'!$B$23)^5</f>
-        <v>1.65248284250861</v>
+        <v>1.66224716105364</v>
       </c>
       <c r="D43" s="67" t="n">
         <f aca="false">D38/(1+'Holdco Summary'!$B$23)^5</f>
-        <v>0.377345072664851</v>
+        <v>0.378286686342777</v>
       </c>
       <c r="E43" s="67" t="n">
         <f aca="false">E38/(1+'Holdco Summary'!$B$23)^5</f>
-        <v>1.29992818408908</v>
+        <v>1.31272785099005</v>
       </c>
       <c r="F43" s="67" t="n">
         <f aca="false">F38/(1+'Holdco Summary'!$B$23)^5</f>
-        <v>1.12471826308982</v>
+        <v>1.13154981031405</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22697,23 +22707,23 @@
       </c>
       <c r="B44" s="46" t="n">
         <f aca="false">(B38/(1+'Holdco Summary'!$B$23)^5)^(1/5)-1</f>
-        <v>0.00440832341012798</v>
+        <v>0.00542344782444015</v>
       </c>
       <c r="C44" s="46" t="n">
         <f aca="false">(C38/(1+'Holdco Summary'!$B$23)^5)^(1/5)-1</f>
-        <v>0.105674749884133</v>
+        <v>0.106978331743751</v>
       </c>
       <c r="D44" s="46" t="n">
         <f aca="false">(D38/(1+'Holdco Summary'!$B$23)^5)^(1/5)-1</f>
-        <v>-0.177098722235455</v>
+        <v>-0.17668844374383</v>
       </c>
       <c r="E44" s="71" t="n">
         <f aca="false">(E38/(1+'Holdco Summary'!$B$23)^5)^(1/5)-1</f>
-        <v>0.053862307970961</v>
+        <v>0.0559295406980851</v>
       </c>
       <c r="F44" s="72" t="n">
         <f aca="false">(F38/(1+'Holdco Summary'!$B$23)^5)^(1/5)-1</f>
-        <v>0.02378496996402</v>
+        <v>0.0250256547711496</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22793,23 +22803,23 @@
       </c>
       <c r="B50" s="62" t="n">
         <f aca="false">'Weapons Sleeve'!C54</f>
-        <v>1296.54096147776</v>
+        <v>1367.85556437661</v>
       </c>
       <c r="C50" s="62" t="n">
         <f aca="false">'Weapons Sleeve'!F54</f>
-        <v>2663.99206233137</v>
+        <v>2817.66321252754</v>
       </c>
       <c r="D50" s="62" t="n">
         <f aca="false">'Weapons Sleeve'!I54</f>
-        <v>451.571462496729</v>
+        <v>465.723649144541</v>
       </c>
       <c r="E50" s="63" t="n">
         <f aca="false">'Weapons Sleeve'!L54</f>
-        <v>2692.9346809097</v>
+        <v>2828.63891069913</v>
       </c>
       <c r="F50" s="64" t="n">
         <f aca="false">B50*'Defense Supercycle'!$B$17+C50*'Defense Supercycle'!$B$18+D50*'Defense Supercycle'!$B$19+E50*'Defense Supercycle'!$B$20</f>
-        <v>1721.1173697588</v>
+        <v>1814.10519107791</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22843,23 +22853,23 @@
       </c>
       <c r="B52" s="66" t="n">
         <f aca="false">B49+B50+B51</f>
-        <v>2736.68600653161</v>
+        <v>2808.00060943046</v>
       </c>
       <c r="C52" s="66" t="n">
         <f aca="false">C49+C50+C51</f>
-        <v>5705.53117688067</v>
+        <v>5859.20232707684</v>
       </c>
       <c r="D52" s="66" t="n">
         <f aca="false">D49+D50+D51</f>
-        <v>700.842397049017</v>
+        <v>714.99458369683</v>
       </c>
       <c r="E52" s="66" t="n">
         <f aca="false">E49+E50+E51</f>
-        <v>4305.56494391885</v>
+        <v>4441.26917370829</v>
       </c>
       <c r="F52" s="66" t="n">
         <f aca="false">F49+F50+F51</f>
-        <v>3408.85259830457</v>
+        <v>3501.84041962368</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22868,23 +22878,23 @@
       </c>
       <c r="B53" s="62" t="n">
         <f aca="false">-'Holdco Summary'!$B$9</f>
-        <v>-840</v>
+        <v>-855</v>
       </c>
       <c r="C53" s="62" t="n">
         <f aca="false">-'Holdco Summary'!$B$9</f>
-        <v>-840</v>
+        <v>-855</v>
       </c>
       <c r="D53" s="62" t="n">
         <f aca="false">-'Holdco Summary'!$B$9</f>
-        <v>-840</v>
+        <v>-855</v>
       </c>
       <c r="E53" s="63" t="n">
         <f aca="false">-'Holdco Summary'!$B$9</f>
-        <v>-840</v>
+        <v>-855</v>
       </c>
       <c r="F53" s="64" t="n">
         <f aca="false">-'Holdco Summary'!$B$9</f>
-        <v>-840</v>
+        <v>-855</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22893,23 +22903,23 @@
       </c>
       <c r="B54" s="62" t="n">
         <f aca="false">-'Holdco Summary'!$B$9*((1+Assumptions!$B$10)^7-1)</f>
-        <v>-599.612385774798</v>
+        <v>-610.31974980649</v>
       </c>
       <c r="C54" s="62" t="n">
         <f aca="false">-'Holdco Summary'!$B$9*((1+Assumptions!$B$10)^7-1)</f>
-        <v>-599.612385774798</v>
+        <v>-610.31974980649</v>
       </c>
       <c r="D54" s="62" t="n">
         <f aca="false">-'Holdco Summary'!$B$9*((1+Assumptions!$B$10)^7-1)</f>
-        <v>-599.612385774798</v>
+        <v>-610.31974980649</v>
       </c>
       <c r="E54" s="63" t="n">
         <f aca="false">-'Holdco Summary'!$B$9*((1+Assumptions!$B$10)^7-1)</f>
-        <v>-599.612385774798</v>
+        <v>-610.31974980649</v>
       </c>
       <c r="F54" s="64" t="n">
         <f aca="false">-'Holdco Summary'!$B$9*((1+Assumptions!$B$10)^7-1)</f>
-        <v>-599.612385774798</v>
+        <v>-610.31974980649</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22918,11 +22928,11 @@
       </c>
       <c r="B55" s="62" t="n">
         <f aca="false">MAX(0,B52+B53+B54)</f>
-        <v>1297.07362075682</v>
+        <v>1342.68085962396</v>
       </c>
       <c r="C55" s="62" t="n">
         <f aca="false">MAX(0,C52+C53+C54)</f>
-        <v>4265.91879110587</v>
+        <v>4393.88257727035</v>
       </c>
       <c r="D55" s="62" t="n">
         <f aca="false">MAX(0,D52+D53+D54)</f>
@@ -22930,11 +22940,11 @@
       </c>
       <c r="E55" s="63" t="n">
         <f aca="false">MAX(0,E52+E53+E54)</f>
-        <v>2865.95255814406</v>
+        <v>2975.9494239018</v>
       </c>
       <c r="F55" s="64" t="n">
         <f aca="false">B55*'Defense Supercycle'!$B$17+C55*'Defense Supercycle'!$B$18+D55*'Defense Supercycle'!$B$19+E55*'Defense Supercycle'!$B$20</f>
-        <v>2080.05571083864</v>
+        <v>2149.06944473364</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22943,11 +22953,11 @@
       </c>
       <c r="B56" s="62" t="n">
         <f aca="false">-Assumptions!$B$9*B55</f>
-        <v>-259.414724151363</v>
+        <v>-268.536171924793</v>
       </c>
       <c r="C56" s="62" t="n">
         <f aca="false">-Assumptions!$B$9*C55</f>
-        <v>-853.183758221174</v>
+        <v>-878.776515454071</v>
       </c>
       <c r="D56" s="62" t="n">
         <f aca="false">-Assumptions!$B$9*D55</f>
@@ -22955,11 +22965,11 @@
       </c>
       <c r="E56" s="63" t="n">
         <f aca="false">-Assumptions!$B$9*E55</f>
-        <v>-573.190511628811</v>
+        <v>-595.189884780359</v>
       </c>
       <c r="F56" s="64" t="n">
         <f aca="false">B56*'Defense Supercycle'!$B$17+C56*'Defense Supercycle'!$B$18+D56*'Defense Supercycle'!$B$19+E56*'Defense Supercycle'!$B$20</f>
-        <v>-416.011142167729</v>
+        <v>-429.813888946728</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22968,23 +22978,23 @@
       </c>
       <c r="B57" s="62" t="n">
         <f aca="false">-'Holdco Summary'!$B$9*Assumptions!$B$8*7</f>
-        <v>-117.6</v>
+        <v>-119.7</v>
       </c>
       <c r="C57" s="62" t="n">
         <f aca="false">-'Holdco Summary'!$B$9*Assumptions!$B$8*7</f>
-        <v>-117.6</v>
+        <v>-119.7</v>
       </c>
       <c r="D57" s="62" t="n">
         <f aca="false">-'Holdco Summary'!$B$9*Assumptions!$B$8*7</f>
-        <v>-117.6</v>
+        <v>-119.7</v>
       </c>
       <c r="E57" s="63" t="n">
         <f aca="false">-'Holdco Summary'!$B$9*Assumptions!$B$8*7</f>
-        <v>-117.6</v>
+        <v>-119.7</v>
       </c>
       <c r="F57" s="64" t="n">
         <f aca="false">-'Holdco Summary'!$B$9*Assumptions!$B$8*7</f>
-        <v>-117.6</v>
+        <v>-119.7</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22993,23 +23003,23 @@
       </c>
       <c r="B58" s="66" t="n">
         <f aca="false">B52+B56+B57</f>
-        <v>2359.67128238025</v>
+        <v>2419.76443750566</v>
       </c>
       <c r="C58" s="66" t="n">
         <f aca="false">C52+C56+C57</f>
-        <v>4734.74741865949</v>
+        <v>4860.72581162277</v>
       </c>
       <c r="D58" s="66" t="n">
         <f aca="false">D52+D56+D57</f>
-        <v>583.242397049017</v>
+        <v>595.29458369683</v>
       </c>
       <c r="E58" s="66" t="n">
         <f aca="false">E52+E56+E57</f>
-        <v>3614.77443229004</v>
+        <v>3726.37928892793</v>
       </c>
       <c r="F58" s="66" t="n">
         <f aca="false">F52+F56+F57</f>
-        <v>2875.24145613685</v>
+        <v>2952.32653067696</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23018,23 +23028,23 @@
       </c>
       <c r="B59" s="67" t="n">
         <f aca="false">B58/'Holdco Summary'!$B$9</f>
-        <v>2.80913247902411</v>
+        <v>2.83013384503586</v>
       </c>
       <c r="C59" s="67" t="n">
         <f aca="false">C58/'Holdco Summary'!$B$9</f>
-        <v>5.63660406983273</v>
+        <v>5.68505942879856</v>
       </c>
       <c r="D59" s="67" t="n">
         <f aca="false">D58/'Holdco Summary'!$B$9</f>
-        <v>0.694336186963116</v>
+        <v>0.696250975084011</v>
       </c>
       <c r="E59" s="67" t="n">
         <f aca="false">E58/'Holdco Summary'!$B$9</f>
-        <v>4.30330289558338</v>
+        <v>4.35833834962331</v>
       </c>
       <c r="F59" s="67" t="n">
         <f aca="false">F58/'Holdco Summary'!$B$9</f>
-        <v>3.42290649540101</v>
+        <v>3.45301348617188</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23043,23 +23053,23 @@
       </c>
       <c r="B60" s="68" t="n">
         <f aca="false">B58/'Holdco Summary'!$B$9</f>
-        <v>2.80913247902411</v>
+        <v>2.83013384503586</v>
       </c>
       <c r="C60" s="68" t="n">
         <f aca="false">C58/'Holdco Summary'!$B$9</f>
-        <v>5.63660406983273</v>
+        <v>5.68505942879856</v>
       </c>
       <c r="D60" s="68" t="n">
         <f aca="false">D58/'Holdco Summary'!$B$9</f>
-        <v>0.694336186963116</v>
+        <v>0.696250975084011</v>
       </c>
       <c r="E60" s="69" t="n">
         <f aca="false">E58/'Holdco Summary'!$B$9</f>
-        <v>4.30330289558338</v>
+        <v>4.35833834962331</v>
       </c>
       <c r="F60" s="70" t="n">
         <f aca="false">F58/'Holdco Summary'!$B$9</f>
-        <v>3.42290649540101</v>
+        <v>3.45301348617188</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23068,23 +23078,23 @@
       </c>
       <c r="B61" s="51" t="n">
         <f aca="false">(B58/'Holdco Summary'!$B$9)^(1/7)-1</f>
-        <v>0.158995489652759</v>
+        <v>0.160229366235885</v>
       </c>
       <c r="C61" s="51" t="n">
         <f aca="false">(C58/'Holdco Summary'!$B$9)^(1/7)-1</f>
-        <v>0.280230644478965</v>
+        <v>0.281797106824369</v>
       </c>
       <c r="D61" s="51" t="n">
         <f aca="false">(D58/'Holdco Summary'!$B$9)^(1/7)-1</f>
-        <v>-0.0507794883216116</v>
+        <v>-0.0504059739765521</v>
       </c>
       <c r="E61" s="51" t="n">
         <f aca="false">(E58/'Holdco Summary'!$B$9)^(1/7)-1</f>
-        <v>0.231808313482553</v>
+        <v>0.234046609741583</v>
       </c>
       <c r="F61" s="51" t="n">
         <f aca="false">(F58/'Holdco Summary'!$B$9)^(1/7)-1</f>
-        <v>0.192180867725363</v>
+        <v>0.193673267252674</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23093,23 +23103,23 @@
       </c>
       <c r="B62" s="68" t="n">
         <f aca="false">B59/(1+'Holdco Summary'!$B$21)^7</f>
-        <v>1.53669166432779</v>
+        <v>1.54818013072471</v>
       </c>
       <c r="C62" s="68" t="n">
         <f aca="false">C59/(1+'Holdco Summary'!$B$21)^7</f>
-        <v>3.08341545082172</v>
+        <v>3.1099221915222</v>
       </c>
       <c r="D62" s="68" t="n">
         <f aca="false">D59/(1+'Holdco Summary'!$B$21)^7</f>
-        <v>0.379825671702756</v>
+        <v>0.380873126376505</v>
       </c>
       <c r="E62" s="69" t="n">
         <f aca="false">E59/(1+'Holdco Summary'!$B$21)^7</f>
-        <v>2.35405404981752</v>
+        <v>2.38416032785786</v>
       </c>
       <c r="F62" s="70" t="n">
         <f aca="false">F59/(1+'Holdco Summary'!$B$21)^7</f>
-        <v>1.87244706988098</v>
+        <v>1.88891662484182</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23118,23 +23128,23 @@
       </c>
       <c r="B63" s="68" t="n">
         <f aca="false">B59/(1+'Holdco Summary'!$B$22)^7</f>
-        <v>1.19405165990218</v>
+        <v>1.20297851405869</v>
       </c>
       <c r="C63" s="68" t="n">
         <f aca="false">C59/(1+'Holdco Summary'!$B$22)^7</f>
-        <v>2.39589855446522</v>
+        <v>2.41649502054019</v>
       </c>
       <c r="D63" s="68" t="n">
         <f aca="false">D59/(1+'Holdco Summary'!$B$22)^7</f>
-        <v>0.295134986606784</v>
+        <v>0.295948887678089</v>
       </c>
       <c r="E63" s="69" t="n">
         <f aca="false">E59/(1+'Holdco Summary'!$B$22)^7</f>
-        <v>1.82916469903131</v>
+        <v>1.85255810455438</v>
       </c>
       <c r="F63" s="70" t="n">
         <f aca="false">F59/(1+'Holdco Summary'!$B$22)^7</f>
-        <v>1.454942838418</v>
+        <v>1.46774013529633</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23143,23 +23153,23 @@
       </c>
       <c r="B64" s="67" t="n">
         <f aca="false">B59/(1+'Holdco Summary'!$B$23)^7</f>
-        <v>1.05605694891614</v>
+        <v>1.06395214028894</v>
       </c>
       <c r="C64" s="67" t="n">
         <f aca="false">C59/(1+'Holdco Summary'!$B$23)^7</f>
-        <v>2.11900824923137</v>
+        <v>2.1372244134494</v>
       </c>
       <c r="D64" s="67" t="n">
         <f aca="false">D59/(1+'Holdco Summary'!$B$23)^7</f>
-        <v>0.261026690838401</v>
+        <v>0.26174653061665</v>
       </c>
       <c r="E64" s="67" t="n">
         <f aca="false">E59/(1+'Holdco Summary'!$B$23)^7</f>
-        <v>1.61777095245809</v>
+        <v>1.63846081814068</v>
       </c>
       <c r="F64" s="67" t="n">
         <f aca="false">F59/(1+'Holdco Summary'!$B$23)^7</f>
-        <v>1.28679733581458</v>
+        <v>1.29811566880597</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23168,23 +23178,23 @@
       </c>
       <c r="B65" s="46" t="n">
         <f aca="false">(B59/(1+'Holdco Summary'!$B$23)^7)^(1/7)-1</f>
-        <v>0.00782216491544263</v>
+        <v>0.00889510107468294</v>
       </c>
       <c r="C65" s="46" t="n">
         <f aca="false">(C59/(1+'Holdco Summary'!$B$23)^7)^(1/7)-1</f>
-        <v>0.113244038677361</v>
+        <v>0.114606179847278</v>
       </c>
       <c r="D65" s="46" t="n">
         <f aca="false">(D59/(1+'Holdco Summary'!$B$23)^7)^(1/7)-1</f>
-        <v>-0.174590859410097</v>
+        <v>-0.174266064327437</v>
       </c>
       <c r="E65" s="71" t="n">
         <f aca="false">(E59/(1+'Holdco Summary'!$B$23)^7)^(1/7)-1</f>
-        <v>0.0711376638978727</v>
+        <v>0.0730840084709419</v>
       </c>
       <c r="F65" s="72" t="n">
         <f aca="false">(F59/(1+'Holdco Summary'!$B$23)^7)^(1/7)-1</f>
-        <v>0.0366790154133589</v>
+        <v>0.0379767541327605</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23264,23 +23274,23 @@
       </c>
       <c r="B71" s="62" t="n">
         <f aca="false">'Weapons Sleeve'!C70</f>
-        <v>2216.90031706174</v>
+        <v>2353.82540279516</v>
       </c>
       <c r="C71" s="62" t="n">
         <f aca="false">'Weapons Sleeve'!F70</f>
-        <v>6362.82597009198</v>
+        <v>6772.83040582878</v>
       </c>
       <c r="D71" s="62" t="n">
         <f aca="false">'Weapons Sleeve'!I70</f>
-        <v>480.983029224514</v>
+        <v>494.569881367072</v>
       </c>
       <c r="E71" s="63" t="n">
         <f aca="false">'Weapons Sleeve'!L70</f>
-        <v>6448.54944420373</v>
+        <v>6791.82840558708</v>
       </c>
       <c r="F71" s="64" t="n">
         <f aca="false">B71*'Defense Supercycle'!$B$17+C71*'Defense Supercycle'!$B$18+D71*'Defense Supercycle'!$B$19+E71*'Defense Supercycle'!$B$20</f>
-        <v>3627.74150621502</v>
+        <v>3845.38877575814</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23314,23 +23324,23 @@
       </c>
       <c r="B73" s="66" t="n">
         <f aca="false">B70+B71+B72</f>
-        <v>4577.67414094336</v>
+        <v>4714.59922667679</v>
       </c>
       <c r="C73" s="66" t="n">
         <f aca="false">C70+C71+C72</f>
-        <v>13290.126985813</v>
+        <v>13700.1314215498</v>
       </c>
       <c r="D73" s="66" t="n">
         <f aca="false">D70+D71+D72</f>
-        <v>691.38298108827</v>
+        <v>704.969833230827</v>
       </c>
       <c r="E73" s="66" t="n">
         <f aca="false">E70+E71+E72</f>
-        <v>9911.87640534353</v>
+        <v>10255.1553667269</v>
       </c>
       <c r="F73" s="66" t="n">
         <f aca="false">F70+F71+F72</f>
-        <v>6972.97401784252</v>
+        <v>7190.62128738565</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23339,23 +23349,23 @@
       </c>
       <c r="B74" s="62" t="n">
         <f aca="false">-'Holdco Summary'!$B$9</f>
-        <v>-840</v>
+        <v>-855</v>
       </c>
       <c r="C74" s="62" t="n">
         <f aca="false">-'Holdco Summary'!$B$9</f>
-        <v>-840</v>
+        <v>-855</v>
       </c>
       <c r="D74" s="62" t="n">
         <f aca="false">-'Holdco Summary'!$B$9</f>
-        <v>-840</v>
+        <v>-855</v>
       </c>
       <c r="E74" s="63" t="n">
         <f aca="false">-'Holdco Summary'!$B$9</f>
-        <v>-840</v>
+        <v>-855</v>
       </c>
       <c r="F74" s="64" t="n">
         <f aca="false">-'Holdco Summary'!$B$9</f>
-        <v>-840</v>
+        <v>-855</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23364,23 +23374,23 @@
       </c>
       <c r="B75" s="62" t="n">
         <f aca="false">-'Holdco Summary'!$B$9*((1+Assumptions!$B$10)^10-1)</f>
-        <v>-973.496997709142</v>
+        <v>-990.880872668234</v>
       </c>
       <c r="C75" s="62" t="n">
         <f aca="false">-'Holdco Summary'!$B$9*((1+Assumptions!$B$10)^10-1)</f>
-        <v>-973.496997709142</v>
+        <v>-990.880872668234</v>
       </c>
       <c r="D75" s="62" t="n">
         <f aca="false">-'Holdco Summary'!$B$9*((1+Assumptions!$B$10)^10-1)</f>
-        <v>-973.496997709142</v>
+        <v>-990.880872668234</v>
       </c>
       <c r="E75" s="63" t="n">
         <f aca="false">-'Holdco Summary'!$B$9*((1+Assumptions!$B$10)^10-1)</f>
-        <v>-973.496997709142</v>
+        <v>-990.880872668234</v>
       </c>
       <c r="F75" s="64" t="n">
         <f aca="false">-'Holdco Summary'!$B$9*((1+Assumptions!$B$10)^10-1)</f>
-        <v>-973.496997709142</v>
+        <v>-990.880872668234</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23389,11 +23399,11 @@
       </c>
       <c r="B76" s="62" t="n">
         <f aca="false">MAX(0,B73+B74+B75)</f>
-        <v>2764.17714323422</v>
+        <v>2868.71835400855</v>
       </c>
       <c r="C76" s="62" t="n">
         <f aca="false">MAX(0,C73+C74+C75)</f>
-        <v>11476.6299881038</v>
+        <v>11854.2505488815</v>
       </c>
       <c r="D76" s="62" t="n">
         <f aca="false">MAX(0,D73+D74+D75)</f>
@@ -23401,11 +23411,11 @@
       </c>
       <c r="E76" s="63" t="n">
         <f aca="false">MAX(0,E73+E74+E75)</f>
-        <v>8098.37940763439</v>
+        <v>8409.27449405865</v>
       </c>
       <c r="F76" s="64" t="n">
         <f aca="false">B76*'Defense Supercycle'!$B$17+C76*'Defense Supercycle'!$B$18+D76*'Defense Supercycle'!$B$19+E76*'Defense Supercycle'!$B$20</f>
-        <v>5327.79412262651</v>
+        <v>5515.87707063303</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23414,11 +23424,11 @@
       </c>
       <c r="B77" s="62" t="n">
         <f aca="false">-Assumptions!$B$9*B76</f>
-        <v>-552.835428646844</v>
+        <v>-573.743670801711</v>
       </c>
       <c r="C77" s="62" t="n">
         <f aca="false">-Assumptions!$B$9*C76</f>
-        <v>-2295.32599762077</v>
+        <v>-2370.85010977631</v>
       </c>
       <c r="D77" s="62" t="n">
         <f aca="false">-Assumptions!$B$9*D76</f>
@@ -23426,11 +23436,11 @@
       </c>
       <c r="E77" s="63" t="n">
         <f aca="false">-Assumptions!$B$9*E76</f>
-        <v>-1619.67588152688</v>
+        <v>-1681.85489881173</v>
       </c>
       <c r="F77" s="64" t="n">
         <f aca="false">B77*'Defense Supercycle'!$B$17+C77*'Defense Supercycle'!$B$18+D77*'Defense Supercycle'!$B$19+E77*'Defense Supercycle'!$B$20</f>
-        <v>-1065.5588245253</v>
+        <v>-1103.17541412661</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23439,23 +23449,23 @@
       </c>
       <c r="B78" s="62" t="n">
         <f aca="false">-'Holdco Summary'!$B$9*Assumptions!$B$8*10</f>
-        <v>-168</v>
+        <v>-171</v>
       </c>
       <c r="C78" s="62" t="n">
         <f aca="false">-'Holdco Summary'!$B$9*Assumptions!$B$8*10</f>
-        <v>-168</v>
+        <v>-171</v>
       </c>
       <c r="D78" s="62" t="n">
         <f aca="false">-'Holdco Summary'!$B$9*Assumptions!$B$8*10</f>
-        <v>-168</v>
+        <v>-171</v>
       </c>
       <c r="E78" s="63" t="n">
         <f aca="false">-'Holdco Summary'!$B$9*Assumptions!$B$8*10</f>
-        <v>-168</v>
+        <v>-171</v>
       </c>
       <c r="F78" s="64" t="n">
         <f aca="false">-'Holdco Summary'!$B$9*Assumptions!$B$8*10</f>
-        <v>-168</v>
+        <v>-171</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23464,23 +23474,23 @@
       </c>
       <c r="B79" s="66" t="n">
         <f aca="false">B73+B77+B78</f>
-        <v>3856.83871229652</v>
+        <v>3969.85555587508</v>
       </c>
       <c r="C79" s="66" t="n">
         <f aca="false">C73+C77+C78</f>
-        <v>10826.8009881922</v>
+        <v>11158.2813117735</v>
       </c>
       <c r="D79" s="66" t="n">
         <f aca="false">D73+D77+D78</f>
-        <v>523.38298108827</v>
+        <v>533.969833230827</v>
       </c>
       <c r="E79" s="66" t="n">
         <f aca="false">E73+E77+E78</f>
-        <v>8124.20052381665</v>
+        <v>8402.30046791515</v>
       </c>
       <c r="F79" s="66" t="n">
         <f aca="false">F73+F77+F78</f>
-        <v>5739.41519331722</v>
+        <v>5916.44587325905</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23489,23 +23499,23 @@
       </c>
       <c r="B80" s="67" t="n">
         <f aca="false">B79/'Holdco Summary'!$B$9</f>
-        <v>4.59147465749586</v>
+        <v>4.64310591330418</v>
       </c>
       <c r="C80" s="67" t="n">
         <f aca="false">C79/'Holdco Summary'!$B$9</f>
-        <v>12.8890487954669</v>
+        <v>13.0506214172789</v>
       </c>
       <c r="D80" s="67" t="n">
         <f aca="false">D79/'Holdco Summary'!$B$9</f>
-        <v>0.623074977486035</v>
+        <v>0.62452612073781</v>
       </c>
       <c r="E80" s="67" t="n">
         <f aca="false">E79/'Holdco Summary'!$B$9</f>
-        <v>9.67166729025792</v>
+        <v>9.82725200925749</v>
       </c>
       <c r="F80" s="67" t="n">
         <f aca="false">F79/'Holdco Summary'!$B$9</f>
-        <v>6.83263713490145</v>
+        <v>6.9198197348059</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23514,23 +23524,23 @@
       </c>
       <c r="B81" s="68" t="n">
         <f aca="false">B79/'Holdco Summary'!$B$9</f>
-        <v>4.59147465749586</v>
+        <v>4.64310591330418</v>
       </c>
       <c r="C81" s="68" t="n">
         <f aca="false">C79/'Holdco Summary'!$B$9</f>
-        <v>12.8890487954669</v>
+        <v>13.0506214172789</v>
       </c>
       <c r="D81" s="68" t="n">
         <f aca="false">D79/'Holdco Summary'!$B$9</f>
-        <v>0.623074977486035</v>
+        <v>0.62452612073781</v>
       </c>
       <c r="E81" s="69" t="n">
         <f aca="false">E79/'Holdco Summary'!$B$9</f>
-        <v>9.67166729025792</v>
+        <v>9.82725200925749</v>
       </c>
       <c r="F81" s="70" t="n">
         <f aca="false">F79/'Holdco Summary'!$B$9</f>
-        <v>6.83263713490145</v>
+        <v>6.9198197348059</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23539,23 +23549,23 @@
       </c>
       <c r="B82" s="51" t="n">
         <f aca="false">(B79/'Holdco Summary'!$B$9)^(1/10)-1</f>
-        <v>0.164649431844847</v>
+        <v>0.165952502895083</v>
       </c>
       <c r="C82" s="51" t="n">
         <f aca="false">(C79/'Holdco Summary'!$B$9)^(1/10)-1</f>
-        <v>0.291284942436493</v>
+        <v>0.292894592849268</v>
       </c>
       <c r="D82" s="51" t="n">
         <f aca="false">(D79/'Holdco Summary'!$B$9)^(1/10)-1</f>
-        <v>-0.0462072190141125</v>
+        <v>-0.045985312895805</v>
       </c>
       <c r="E82" s="51" t="n">
         <f aca="false">(E79/'Holdco Summary'!$B$9)^(1/10)-1</f>
-        <v>0.25472957508494</v>
+        <v>0.256733550220737</v>
       </c>
       <c r="F82" s="51" t="n">
         <f aca="false">(F79/'Holdco Summary'!$B$9)^(1/10)-1</f>
-        <v>0.211877816332995</v>
+        <v>0.213415331908954</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23564,23 +23574,23 @@
       </c>
       <c r="B83" s="68" t="n">
         <f aca="false">B80/(1+'Holdco Summary'!$B$21)^10</f>
-        <v>1.93948851491393</v>
+        <v>1.96129811534096</v>
       </c>
       <c r="C83" s="68" t="n">
         <f aca="false">C80/(1+'Holdco Summary'!$B$21)^10</f>
-        <v>5.44447350181108</v>
+        <v>5.51272352336294</v>
       </c>
       <c r="D83" s="68" t="n">
         <f aca="false">D80/(1+'Holdco Summary'!$B$21)^10</f>
-        <v>0.263193603996389</v>
+        <v>0.263806582588293</v>
       </c>
       <c r="E83" s="69" t="n">
         <f aca="false">E80/(1+'Holdco Summary'!$B$21)^10</f>
-        <v>4.08541678410449</v>
+        <v>4.15113745079773</v>
       </c>
       <c r="F83" s="70" t="n">
         <f aca="false">F80/(1+'Holdco Summary'!$B$21)^10</f>
-        <v>2.88617976537917</v>
+        <v>2.92300663775207</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23589,23 +23599,23 @@
       </c>
       <c r="B84" s="68" t="n">
         <f aca="false">B80/(1+'Holdco Summary'!$B$22)^10</f>
-        <v>1.35259493481467</v>
+        <v>1.36780490117492</v>
       </c>
       <c r="C84" s="68" t="n">
         <f aca="false">C80/(1+'Holdco Summary'!$B$22)^10</f>
-        <v>3.79696359357363</v>
+        <v>3.84456100533563</v>
       </c>
       <c r="D84" s="68" t="n">
         <f aca="false">D80/(1+'Holdco Summary'!$B$22)^10</f>
-        <v>0.183550628376334</v>
+        <v>0.183978118269769</v>
       </c>
       <c r="E84" s="69" t="n">
         <f aca="false">E80/(1+'Holdco Summary'!$B$22)^10</f>
-        <v>2.84916049066256</v>
+        <v>2.89499393602631</v>
       </c>
       <c r="F84" s="70" t="n">
         <f aca="false">F80/(1+'Holdco Summary'!$B$22)^10</f>
-        <v>2.01281528691584</v>
+        <v>2.03849826500703</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23614,23 +23624,23 @@
       </c>
       <c r="B85" s="67" t="n">
         <f aca="false">B80/(1+'Holdco Summary'!$B$23)^10</f>
-        <v>1.13494231387911</v>
+        <v>1.14770477067279</v>
       </c>
       <c r="C85" s="67" t="n">
         <f aca="false">C80/(1+'Holdco Summary'!$B$23)^10</f>
-        <v>3.18597573869788</v>
+        <v>3.22591401973781</v>
       </c>
       <c r="D85" s="67" t="n">
         <f aca="false">D80/(1+'Holdco Summary'!$B$23)^10</f>
-        <v>0.154014605201774</v>
+        <v>0.154373305620004</v>
       </c>
       <c r="E85" s="67" t="n">
         <f aca="false">E80/(1+'Holdco Summary'!$B$23)^10</f>
-        <v>2.39068823685087</v>
+        <v>2.42914639989383</v>
       </c>
       <c r="F85" s="67" t="n">
         <f aca="false">F80/(1+'Holdco Summary'!$B$23)^10</f>
-        <v>1.68892340222796</v>
+        <v>1.71047360756428</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23639,23 +23649,23 @@
       </c>
       <c r="B86" s="46" t="n">
         <f aca="false">(B80/(1+'Holdco Summary'!$B$23)^10)^(1/10)-1</f>
-        <v>0.0127386363868236</v>
+        <v>0.0138717416478982</v>
       </c>
       <c r="C86" s="46" t="n">
         <f aca="false">(C80/(1+'Holdco Summary'!$B$23)^10)^(1/10)-1</f>
-        <v>0.122856471683907</v>
+        <v>0.124256167695016</v>
       </c>
       <c r="D86" s="46" t="n">
         <f aca="false">(D80/(1+'Holdco Summary'!$B$23)^10)^(1/10)-1</f>
-        <v>-0.17061497305575</v>
+        <v>-0.170422011213743</v>
       </c>
       <c r="E86" s="71" t="n">
         <f aca="false">(E80/(1+'Holdco Summary'!$B$23)^10)^(1/10)-1</f>
-        <v>0.0910691957260348</v>
+        <v>0.0928117828006405</v>
       </c>
       <c r="F86" s="72" t="n">
         <f aca="false">(F80/(1+'Holdco Summary'!$B$23)^10)^(1/10)-1</f>
-        <v>0.0538067968112996</v>
+        <v>0.0551437668773511</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -23743,6 +23753,7 @@
     <oddHeader/>
     <oddFooter>&amp;LLeviathan Core PE Holdco — Internal / Confidential&amp;R&amp;A  |  Page &amp;P of &amp;N</oddFooter>
   </headerFooter>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 

</xml_diff>